<commit_message>
Spreadsheet: add asset sizes and a Measurements sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BBz4kUXe8DBQeVKEZD3dJv
</commit_message>
<xml_diff>
--- a/docs/Derelict-Mill-Alley-Tracker.xlsx
+++ b/docs/Derelict-Mill-Alley-Tracker.xlsx
@@ -4,6 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mill Alley" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
     <numFmt numFmtId="166" formatCode="ddd m/d"/>
     <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -46,6 +47,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="FF555555"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <i val="1"/>
       <color rgb="FF666666"/>
       <sz val="9"/>
@@ -61,8 +67,13 @@
       <color rgb="FF999999"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -135,6 +146,11 @@
         <fgColor rgb="FFCCCCCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEF3F4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -142,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -203,30 +219,41 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1013,7 +1040,7 @@
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="34" customWidth="1" style="17" min="1" max="1"/>
-    <col width="12" customWidth="1" style="17" min="2" max="2"/>
+    <col width="26" customWidth="1" style="17" min="2" max="2"/>
     <col width="7.5" customWidth="1" style="17" min="3" max="3"/>
     <col width="5.88" customWidth="1" style="17" min="4" max="4"/>
     <col width="7.63" customWidth="1" style="17" min="5" max="5"/>
@@ -1047,7 +1074,11 @@
           <t>Kit A · Left mill</t>
         </is>
       </c>
-      <c r="B2" s="19" t="n"/>
+      <c r="B2" s="19" t="inlineStr">
+        <is>
+          <t>Size (cm)</t>
+        </is>
+      </c>
       <c r="C2" s="19" t="inlineStr">
         <is>
           <t>Blockout</t>
@@ -1121,43 +1152,47 @@
           <t>A01 Wall flat</t>
         </is>
       </c>
-      <c r="B4" s="8" t="n"/>
-      <c r="C4" s="24" t="n"/>
-      <c r="D4" s="24" t="n"/>
-      <c r="E4" s="24" t="n"/>
-      <c r="F4" s="24" t="n"/>
-      <c r="G4" s="24" t="n"/>
-      <c r="I4" s="25" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>400 x 400, 200 x 400, 100 x 400</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="n"/>
+      <c r="D4" s="25" t="n"/>
+      <c r="E4" s="25" t="n"/>
+      <c r="F4" s="25" t="n"/>
+      <c r="G4" s="25" t="n"/>
+      <c r="I4" s="26" t="inlineStr">
         <is>
           <t>Build a reference board</t>
         </is>
       </c>
-      <c r="J4" s="25" t="inlineStr">
+      <c r="J4" s="26" t="inlineStr">
         <is>
           <t>Paint over the reference</t>
         </is>
       </c>
-      <c r="K4" s="26" t="inlineStr">
+      <c r="K4" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="L4" s="26" t="inlineStr">
+      <c r="L4" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="M4" s="25" t="inlineStr">
+      <c r="M4" s="26" t="inlineStr">
         <is>
           <t>Camera match in Blender</t>
         </is>
       </c>
-      <c r="N4" s="25" t="inlineStr">
+      <c r="N4" s="26" t="inlineStr">
         <is>
           <t>Lock metrics, naming and folders</t>
         </is>
       </c>
-      <c r="O4" s="25" t="inlineStr">
+      <c r="O4" s="26" t="inlineStr">
         <is>
           <t>Lighting and mood paintover + Review 1</t>
         </is>
@@ -1169,19 +1204,23 @@
           <t>A02 Pilaster</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="24" t="n"/>
-      <c r="D5" s="24" t="n"/>
-      <c r="E5" s="24" t="n"/>
-      <c r="F5" s="24" t="n"/>
-      <c r="G5" s="24" t="n"/>
-      <c r="I5" s="27" t="n"/>
-      <c r="J5" s="27" t="n"/>
-      <c r="K5" s="27" t="n"/>
-      <c r="L5" s="27" t="n"/>
-      <c r="M5" s="27" t="n"/>
-      <c r="N5" s="27" t="n"/>
-      <c r="O5" s="27" t="n"/>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>60 x 400, 25 projection</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="n"/>
+      <c r="D5" s="25" t="n"/>
+      <c r="E5" s="25" t="n"/>
+      <c r="F5" s="25" t="n"/>
+      <c r="G5" s="25" t="n"/>
+      <c r="I5" s="28" t="n"/>
+      <c r="J5" s="28" t="n"/>
+      <c r="K5" s="28" t="n"/>
+      <c r="L5" s="28" t="n"/>
+      <c r="M5" s="28" t="n"/>
+      <c r="N5" s="28" t="n"/>
+      <c r="O5" s="28" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="23" t="inlineStr">
@@ -1189,12 +1228,16 @@
           <t>A03 Blind arch recess with brick infill</t>
         </is>
       </c>
-      <c r="B6" s="8" t="n"/>
-      <c r="C6" s="24" t="n"/>
-      <c r="D6" s="24" t="n"/>
-      <c r="E6" s="24" t="n"/>
-      <c r="F6" s="24" t="n"/>
-      <c r="G6" s="24" t="n"/>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>300 x 600</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="n"/>
+      <c r="D6" s="25" t="n"/>
+      <c r="E6" s="25" t="n"/>
+      <c r="F6" s="25" t="n"/>
+      <c r="G6" s="25" t="n"/>
       <c r="I6" s="19" t="inlineStr">
         <is>
           <t>Week 2 · Greybox</t>
@@ -1213,12 +1256,16 @@
           <t>A04 Upper window, round head, glazed</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="24" t="n"/>
-      <c r="D7" s="24" t="n"/>
-      <c r="E7" s="24" t="n"/>
-      <c r="F7" s="24" t="n"/>
-      <c r="G7" s="24" t="n"/>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>300 x 400</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="n"/>
+      <c r="D7" s="25" t="n"/>
+      <c r="E7" s="25" t="n"/>
+      <c r="F7" s="25" t="n"/>
+      <c r="G7" s="25" t="n"/>
       <c r="I7" s="22" t="n">
         <v>46321</v>
       </c>
@@ -1247,43 +1294,47 @@
           <t>A05 Arched loading door surround</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="24" t="n"/>
-      <c r="D8" s="24" t="n"/>
-      <c r="E8" s="24" t="n"/>
-      <c r="F8" s="24" t="n"/>
-      <c r="G8" s="24" t="n"/>
-      <c r="I8" s="25" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>300 x 400</t>
+        </is>
+      </c>
+      <c r="C8" s="25" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
+      <c r="F8" s="25" t="n"/>
+      <c r="G8" s="25" t="n"/>
+      <c r="I8" s="26" t="inlineStr">
         <is>
           <t>Greybox ground and both building masses in UE5 at scale</t>
         </is>
       </c>
-      <c r="J8" s="25" t="inlineStr">
+      <c r="J8" s="26" t="inlineStr">
         <is>
           <t>Greybox the left facade with placeholder A01 to A09 at final dimensions</t>
         </is>
       </c>
-      <c r="K8" s="26" t="inlineStr">
+      <c r="K8" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="L8" s="26" t="inlineStr">
+      <c r="L8" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="M8" s="25" t="inlineStr">
+      <c r="M8" s="26" t="inlineStr">
         <is>
           <t>Greybox the right facade with B01 to B09, including the ledge and light well</t>
         </is>
       </c>
-      <c r="N8" s="25" t="inlineStr">
+      <c r="N8" s="26" t="inlineStr">
         <is>
           <t>Greybox skybridge, chimney, end building and loading door</t>
         </is>
       </c>
-      <c r="O8" s="25" t="inlineStr">
+      <c r="O8" s="26" t="inlineStr">
         <is>
           <t>Blockout lighting + Review 2</t>
         </is>
@@ -1296,18 +1347,23 @@
           <t>A06 Outer and inner corner</t>
         </is>
       </c>
-      <c r="C9" s="24" t="n"/>
-      <c r="D9" s="24" t="n"/>
-      <c r="E9" s="24" t="n"/>
-      <c r="F9" s="24" t="n"/>
-      <c r="G9" s="24" t="n"/>
-      <c r="I9" s="27" t="n"/>
-      <c r="J9" s="27" t="n"/>
-      <c r="K9" s="27" t="n"/>
-      <c r="L9" s="27" t="n"/>
-      <c r="M9" s="27" t="n"/>
-      <c r="N9" s="27" t="n"/>
-      <c r="O9" s="27" t="n"/>
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>50 x 400</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="n"/>
+      <c r="D9" s="25" t="n"/>
+      <c r="E9" s="25" t="n"/>
+      <c r="F9" s="25" t="n"/>
+      <c r="G9" s="25" t="n"/>
+      <c r="I9" s="28" t="n"/>
+      <c r="J9" s="28" t="n"/>
+      <c r="K9" s="28" t="n"/>
+      <c r="L9" s="28" t="n"/>
+      <c r="M9" s="28" t="n"/>
+      <c r="N9" s="28" t="n"/>
+      <c r="O9" s="28" t="n"/>
       <c r="Q9" s="8" t="n"/>
     </row>
     <row r="10">
@@ -1316,11 +1372,16 @@
           <t>A07 String course</t>
         </is>
       </c>
-      <c r="C10" s="24" t="n"/>
-      <c r="D10" s="24" t="n"/>
-      <c r="E10" s="24" t="n"/>
-      <c r="F10" s="24" t="n"/>
-      <c r="G10" s="24" t="n"/>
+      <c r="B10" s="29" t="inlineStr">
+        <is>
+          <t>400 long</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="n"/>
+      <c r="D10" s="25" t="n"/>
+      <c r="E10" s="25" t="n"/>
+      <c r="F10" s="25" t="n"/>
+      <c r="G10" s="25" t="n"/>
       <c r="I10" s="19" t="inlineStr">
         <is>
           <t>Week 3 · Tiling materials</t>
@@ -1334,16 +1395,21 @@
       <c r="O10" s="19" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t>A08 Parapet with coping</t>
         </is>
       </c>
-      <c r="C11" s="24" t="n"/>
-      <c r="D11" s="24" t="n"/>
-      <c r="E11" s="24" t="n"/>
-      <c r="F11" s="24" t="n"/>
-      <c r="G11" s="24" t="n"/>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>400 x 100</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="n"/>
+      <c r="D11" s="25" t="n"/>
+      <c r="E11" s="25" t="n"/>
+      <c r="F11" s="25" t="n"/>
+      <c r="G11" s="25" t="n"/>
       <c r="I11" s="22" t="n">
         <v>46328</v>
       </c>
@@ -1367,47 +1433,52 @@
       </c>
     </row>
     <row r="12" ht="58" customHeight="1" s="17">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="30" t="inlineStr">
         <is>
           <t>A09 Base course / plinth</t>
         </is>
       </c>
-      <c r="C12" s="24" t="n"/>
-      <c r="D12" s="24" t="n"/>
-      <c r="E12" s="24" t="n"/>
-      <c r="F12" s="24" t="n"/>
-      <c r="G12" s="24" t="n"/>
-      <c r="I12" s="25" t="inlineStr">
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>400 x 60</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="n"/>
+      <c r="D12" s="25" t="n"/>
+      <c r="E12" s="25" t="n"/>
+      <c r="F12" s="25" t="n"/>
+      <c r="G12" s="25" t="n"/>
+      <c r="I12" s="26" t="inlineStr">
         <is>
           <t>Source CC0 base materials</t>
         </is>
       </c>
-      <c r="J12" s="25" t="inlineStr">
+      <c r="J12" s="26" t="inlineStr">
         <is>
           <t>Build custom mask node groups in Blender</t>
         </is>
       </c>
-      <c r="K12" s="26" t="inlineStr">
+      <c r="K12" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="L12" s="26" t="inlineStr">
+      <c r="L12" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="M12" s="25" t="inlineStr">
+      <c r="M12" s="26" t="inlineStr">
         <is>
           <t>Brick sets M01 to M04</t>
         </is>
       </c>
-      <c r="N12" s="25" t="inlineStr">
+      <c r="N12" s="26" t="inlineStr">
         <is>
           <t>M05 to M10</t>
         </is>
       </c>
-      <c r="O12" s="25" t="inlineStr">
+      <c r="O12" s="26" t="inlineStr">
         <is>
           <t>Build M_Master_Kit in UE5 + Review 3</t>
         </is>
@@ -1415,12 +1486,16 @@
       <c r="P12" s="14" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>Kit B · Right building</t>
         </is>
       </c>
-      <c r="B13" s="29" t="n"/>
+      <c r="B13" s="31" t="inlineStr">
+        <is>
+          <t>Size (cm)</t>
+        </is>
+      </c>
       <c r="C13" s="19" t="inlineStr">
         <is>
           <t>Blockout</t>
@@ -1446,18 +1521,18 @@
           <t>In UE5</t>
         </is>
       </c>
-      <c r="I13" s="27" t="n"/>
-      <c r="J13" s="27" t="n"/>
-      <c r="K13" s="27" t="n"/>
-      <c r="L13" s="27" t="n"/>
-      <c r="M13" s="27" t="n"/>
-      <c r="N13" s="27" t="n"/>
-      <c r="O13" s="27" t="n"/>
+      <c r="I13" s="28" t="n"/>
+      <c r="J13" s="28" t="n"/>
+      <c r="K13" s="28" t="n"/>
+      <c r="L13" s="28" t="n"/>
+      <c r="M13" s="28" t="n"/>
+      <c r="N13" s="28" t="n"/>
+      <c r="O13" s="28" t="n"/>
       <c r="P13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="30" t="n"/>
-      <c r="B14" s="30" t="n"/>
+      <c r="A14" s="32" t="n"/>
+      <c r="B14" s="32" t="n"/>
       <c r="C14" s="21" t="n"/>
       <c r="D14" s="21" t="n"/>
       <c r="E14" s="21" t="n"/>
@@ -1476,16 +1551,21 @@
       <c r="O14" s="19" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="30" t="inlineStr">
         <is>
           <t>B01 Wall flat, painted</t>
         </is>
       </c>
-      <c r="C15" s="24" t="n"/>
-      <c r="D15" s="24" t="n"/>
-      <c r="E15" s="24" t="n"/>
-      <c r="F15" s="24" t="n"/>
-      <c r="G15" s="24" t="n"/>
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>400 x 380, 200 x 380, 100 x 380</t>
+        </is>
+      </c>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
       <c r="I15" s="22" t="n">
         <v>46335</v>
       </c>
@@ -1514,79 +1594,92 @@
           <t>B02 Window bay (opening, sill, lintel)</t>
         </is>
       </c>
-      <c r="B16" s="8" t="n"/>
-      <c r="C16" s="24" t="n"/>
-      <c r="D16" s="24" t="n"/>
-      <c r="E16" s="24" t="n"/>
-      <c r="F16" s="24" t="n"/>
-      <c r="G16" s="24" t="n"/>
-      <c r="I16" s="25" t="inlineStr">
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>300 x 380</t>
+        </is>
+      </c>
+      <c r="C16" s="25" t="n"/>
+      <c r="D16" s="25" t="n"/>
+      <c r="E16" s="25" t="n"/>
+      <c r="F16" s="25" t="n"/>
+      <c r="G16" s="25" t="n"/>
+      <c r="I16" s="26" t="inlineStr">
         <is>
           <t>Model T01 stone and T02 metal trim strips in Blender</t>
         </is>
       </c>
-      <c r="J16" s="25" t="inlineStr">
+      <c r="J16" s="26" t="inlineStr">
         <is>
           <t>T03 timber trim sheet</t>
         </is>
       </c>
-      <c r="K16" s="26" t="inlineStr">
+      <c r="K16" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="L16" s="26" t="inlineStr">
+      <c r="L16" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="M16" s="25" t="inlineStr">
+      <c r="M16" s="26" t="inlineStr">
         <is>
           <t>Model A01, A02, A06, A09 with bevels and UVs</t>
         </is>
       </c>
-      <c r="N16" s="25" t="inlineStr">
+      <c r="N16" s="26" t="inlineStr">
         <is>
           <t>Model A03 blind arch with infill, A05 door surround, A07 string course, A08 parapet</t>
         </is>
       </c>
-      <c r="O16" s="25" t="inlineStr">
+      <c r="O16" s="26" t="inlineStr">
         <is>
           <t>Model A04 window + Review 4</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="31" t="inlineStr">
+      <c r="A17" s="33" t="inlineStr">
         <is>
           <t>B03 Steel window insert: intact, broken, gutted</t>
         </is>
       </c>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="24" t="n"/>
-      <c r="D17" s="24" t="n"/>
-      <c r="E17" s="24" t="n"/>
-      <c r="F17" s="24" t="n"/>
-      <c r="G17" s="24" t="n"/>
-      <c r="I17" s="27" t="n"/>
-      <c r="J17" s="27" t="n"/>
-      <c r="K17" s="27" t="n"/>
-      <c r="L17" s="27" t="n"/>
-      <c r="M17" s="27" t="n"/>
-      <c r="N17" s="27" t="n"/>
-      <c r="O17" s="27" t="n"/>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>140 x 220</t>
+        </is>
+      </c>
+      <c r="C17" s="25" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="I17" s="28" t="n"/>
+      <c r="J17" s="28" t="n"/>
+      <c r="K17" s="28" t="n"/>
+      <c r="L17" s="28" t="n"/>
+      <c r="M17" s="28" t="n"/>
+      <c r="N17" s="28" t="n"/>
+      <c r="O17" s="28" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="28" t="inlineStr">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>B04 Door bay with timber door</t>
         </is>
       </c>
-      <c r="C18" s="24" t="n"/>
-      <c r="D18" s="24" t="n"/>
-      <c r="E18" s="24" t="n"/>
-      <c r="F18" s="24" t="n"/>
-      <c r="G18" s="24" t="n"/>
+      <c r="B18" s="29" t="inlineStr">
+        <is>
+          <t>300 x 380</t>
+        </is>
+      </c>
+      <c r="C18" s="25" t="n"/>
+      <c r="D18" s="25" t="n"/>
+      <c r="E18" s="25" t="n"/>
+      <c r="F18" s="25" t="n"/>
+      <c r="G18" s="25" t="n"/>
       <c r="I18" s="19" t="inlineStr">
         <is>
           <t>Week 5 · Families B, C and D</t>
@@ -1600,16 +1693,21 @@
       <c r="O18" s="19" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="30" t="inlineStr">
         <is>
           <t>B05 Projecting ledge / plinth</t>
         </is>
       </c>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="24" t="n"/>
-      <c r="E19" s="24" t="n"/>
-      <c r="F19" s="24" t="n"/>
-      <c r="G19" s="24" t="n"/>
+      <c r="B19" s="29" t="inlineStr">
+        <is>
+          <t>400 x 50, 60 deep</t>
+        </is>
+      </c>
+      <c r="C19" s="25" t="n"/>
+      <c r="D19" s="25" t="n"/>
+      <c r="E19" s="25" t="n"/>
+      <c r="F19" s="25" t="n"/>
+      <c r="G19" s="25" t="n"/>
       <c r="I19" s="22" t="n">
         <v>46342</v>
       </c>
@@ -1638,78 +1736,92 @@
           <t>B06 Light well: walls, steps, landing</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n"/>
-      <c r="C20" s="24" t="n"/>
-      <c r="D20" s="24" t="n"/>
-      <c r="E20" s="24" t="n"/>
-      <c r="F20" s="24" t="n"/>
-      <c r="G20" s="24" t="n"/>
-      <c r="I20" s="25" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>120 x 380, 200 drop</t>
+        </is>
+      </c>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="I20" s="26" t="inlineStr">
         <is>
           <t>Model B01, B07, B08, B09</t>
         </is>
       </c>
-      <c r="J20" s="25" t="inlineStr">
+      <c r="J20" s="26" t="inlineStr">
         <is>
           <t>Model B02 window bay and the three B03 steel window variants</t>
         </is>
       </c>
-      <c r="K20" s="26" t="inlineStr">
+      <c r="K20" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="L20" s="26" t="inlineStr">
+      <c r="L20" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="M20" s="25" t="inlineStr">
+      <c r="M20" s="26" t="inlineStr">
         <is>
           <t>Model B04 door bay, B05 ledge, B06 light well</t>
         </is>
       </c>
-      <c r="N20" s="25" t="inlineStr">
+      <c r="N20" s="26" t="inlineStr">
         <is>
           <t>Model Family C</t>
         </is>
       </c>
-      <c r="O20" s="25" t="inlineStr">
+      <c r="O20" s="26" t="inlineStr">
         <is>
           <t>Model Family D ground pieces + Review 5</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="28" t="inlineStr">
+      <c r="A21" s="30" t="inlineStr">
         <is>
           <t>B07 Floor band</t>
         </is>
       </c>
-      <c r="C21" s="24" t="n"/>
-      <c r="D21" s="24" t="n"/>
-      <c r="E21" s="24" t="n"/>
-      <c r="F21" s="24" t="n"/>
-      <c r="G21" s="24" t="n"/>
-      <c r="I21" s="27" t="n"/>
-      <c r="J21" s="27" t="n"/>
-      <c r="K21" s="27" t="n"/>
-      <c r="L21" s="27" t="n"/>
-      <c r="M21" s="27" t="n"/>
-      <c r="N21" s="27" t="n"/>
-      <c r="O21" s="27" t="n"/>
+      <c r="B21" s="29" t="inlineStr">
+        <is>
+          <t>400 long</t>
+        </is>
+      </c>
+      <c r="C21" s="25" t="n"/>
+      <c r="D21" s="25" t="n"/>
+      <c r="E21" s="25" t="n"/>
+      <c r="F21" s="25" t="n"/>
+      <c r="G21" s="25" t="n"/>
+      <c r="I21" s="28" t="n"/>
+      <c r="J21" s="28" t="n"/>
+      <c r="K21" s="28" t="n"/>
+      <c r="L21" s="28" t="n"/>
+      <c r="M21" s="28" t="n"/>
+      <c r="N21" s="28" t="n"/>
+      <c r="O21" s="28" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="28" t="inlineStr">
+      <c r="A22" s="30" t="inlineStr">
         <is>
           <t>B08 Outer corner</t>
         </is>
       </c>
-      <c r="C22" s="24" t="n"/>
-      <c r="D22" s="24" t="n"/>
-      <c r="E22" s="24" t="n"/>
-      <c r="F22" s="24" t="n"/>
-      <c r="G22" s="24" t="n"/>
+      <c r="B22" s="29" t="inlineStr">
+        <is>
+          <t>50 x 380</t>
+        </is>
+      </c>
+      <c r="C22" s="25" t="n"/>
+      <c r="D22" s="25" t="n"/>
+      <c r="E22" s="25" t="n"/>
+      <c r="F22" s="25" t="n"/>
+      <c r="G22" s="25" t="n"/>
       <c r="I22" s="19" t="inlineStr">
         <is>
           <t>Week 6 · Hero: skybridge (H1)</t>
@@ -1728,12 +1840,16 @@
           <t>B09 Roof edge with gutter</t>
         </is>
       </c>
-      <c r="B23" s="8" t="n"/>
-      <c r="C23" s="24" t="n"/>
-      <c r="D23" s="24" t="n"/>
-      <c r="E23" s="24" t="n"/>
-      <c r="F23" s="24" t="n"/>
-      <c r="G23" s="24" t="n"/>
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>400 long</t>
+        </is>
+      </c>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
       <c r="I23" s="22" t="n">
         <v>46349</v>
       </c>
@@ -1762,7 +1878,11 @@
           <t>Kit C · Structure</t>
         </is>
       </c>
-      <c r="B24" s="19" t="n"/>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>Size (cm)</t>
+        </is>
+      </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
           <t>Blockout</t>
@@ -1788,69 +1908,74 @@
           <t>In UE5</t>
         </is>
       </c>
-      <c r="I24" s="25" t="inlineStr">
+      <c r="I24" s="26" t="inlineStr">
         <is>
           <t>Plan the skybridge from reference</t>
         </is>
       </c>
-      <c r="J24" s="25" t="inlineStr">
+      <c r="J24" s="26" t="inlineStr">
         <is>
           <t>Sculpt in Blender</t>
         </is>
       </c>
-      <c r="K24" s="26" t="inlineStr">
+      <c r="K24" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="L24" s="26" t="inlineStr">
+      <c r="L24" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="M24" s="25" t="inlineStr">
+      <c r="M24" s="26" t="inlineStr">
         <is>
           <t>Retopo the low poly, UV into two 4K sets</t>
         </is>
       </c>
-      <c r="N24" s="25" t="inlineStr">
+      <c r="N24" s="26" t="inlineStr">
         <is>
           <t>Bake in Marmoset</t>
         </is>
       </c>
-      <c r="O24" s="25" t="inlineStr">
+      <c r="O24" s="26" t="inlineStr">
         <is>
           <t>Finish texturing, import, place + Review 6</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="30" t="n"/>
-      <c r="B25" s="30" t="n"/>
+      <c r="A25" s="32" t="n"/>
+      <c r="B25" s="32" t="n"/>
       <c r="C25" s="21" t="n"/>
       <c r="D25" s="21" t="n"/>
       <c r="E25" s="21" t="n"/>
       <c r="F25" s="21" t="n"/>
       <c r="G25" s="21" t="n"/>
-      <c r="I25" s="27" t="n"/>
-      <c r="J25" s="27" t="n"/>
-      <c r="K25" s="27" t="n"/>
-      <c r="L25" s="27" t="n"/>
-      <c r="M25" s="27" t="n"/>
-      <c r="N25" s="27" t="n"/>
-      <c r="O25" s="27" t="n"/>
+      <c r="I25" s="28" t="n"/>
+      <c r="J25" s="28" t="n"/>
+      <c r="K25" s="28" t="n"/>
+      <c r="L25" s="28" t="n"/>
+      <c r="M25" s="28" t="n"/>
+      <c r="N25" s="28" t="n"/>
+      <c r="O25" s="28" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="28" t="inlineStr">
+      <c r="A26" s="30" t="inlineStr">
         <is>
           <t>C01 Steel I-beam</t>
         </is>
       </c>
-      <c r="C26" s="24" t="n"/>
-      <c r="D26" s="24" t="n"/>
-      <c r="E26" s="24" t="n"/>
-      <c r="F26" s="24" t="n"/>
-      <c r="G26" s="24" t="n"/>
+      <c r="B26" s="29" t="inlineStr">
+        <is>
+          <t>100, 200, 400 long, 30 deep</t>
+        </is>
+      </c>
+      <c r="C26" s="25" t="n"/>
+      <c r="D26" s="25" t="n"/>
+      <c r="E26" s="25" t="n"/>
+      <c r="F26" s="25" t="n"/>
+      <c r="G26" s="25" t="n"/>
       <c r="I26" s="19" t="inlineStr">
         <is>
           <t>Week 7 · Heroes H2, H3, H6, H7</t>
@@ -1864,16 +1989,21 @@
       <c r="O26" s="19" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="28" t="inlineStr">
+      <c r="A27" s="30" t="inlineStr">
         <is>
           <t>C02 Drainpipe: straight, elbow, offset, shoe</t>
         </is>
       </c>
-      <c r="C27" s="24" t="n"/>
-      <c r="D27" s="24" t="n"/>
-      <c r="E27" s="24" t="n"/>
-      <c r="F27" s="24" t="n"/>
-      <c r="G27" s="24" t="n"/>
+      <c r="B27" s="29" t="inlineStr">
+        <is>
+          <t>100, 200, 400; 10 diameter</t>
+        </is>
+      </c>
+      <c r="C27" s="25" t="n"/>
+      <c r="D27" s="25" t="n"/>
+      <c r="E27" s="25" t="n"/>
+      <c r="F27" s="25" t="n"/>
+      <c r="G27" s="25" t="n"/>
       <c r="I27" s="22" t="n">
         <v>46356</v>
       </c>
@@ -1902,67 +2032,75 @@
           <t>C03 Hopper head</t>
         </is>
       </c>
-      <c r="B28" s="8" t="n"/>
-      <c r="C28" s="24" t="n"/>
-      <c r="D28" s="24" t="n"/>
-      <c r="E28" s="24" t="n"/>
-      <c r="F28" s="24" t="n"/>
-      <c r="G28" s="24" t="n"/>
-      <c r="I28" s="25" t="inlineStr">
+      <c r="B28" s="24" t="inlineStr">
+        <is>
+          <t>30 x 30</t>
+        </is>
+      </c>
+      <c r="C28" s="25" t="n"/>
+      <c r="D28" s="25" t="n"/>
+      <c r="E28" s="25" t="n"/>
+      <c r="F28" s="25" t="n"/>
+      <c r="G28" s="25" t="n"/>
+      <c r="I28" s="26" t="inlineStr">
         <is>
           <t>Model the chimney and red end building</t>
         </is>
       </c>
-      <c r="J28" s="25" t="inlineStr">
+      <c r="J28" s="26" t="inlineStr">
         <is>
           <t>Texture the chimney cap</t>
         </is>
       </c>
-      <c r="K28" s="26" t="inlineStr">
+      <c r="K28" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="L28" s="26" t="inlineStr">
+      <c r="L28" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="M28" s="25" t="inlineStr">
+      <c r="M28" s="26" t="inlineStr">
         <is>
           <t>H7 broken glazing variants and M_Master_Glass + Review 7</t>
         </is>
       </c>
-      <c r="N28" s="32" t="inlineStr">
+      <c r="N28" s="34" t="inlineStr">
         <is>
           <t>Buffer: catch up on anything late from Weeks 3 to 7</t>
         </is>
       </c>
-      <c r="O28" s="32" t="inlineStr">
+      <c r="O28" s="34" t="inlineStr">
         <is>
           <t>Buffer</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="31" t="inlineStr">
+      <c r="A29" s="33" t="inlineStr">
         <is>
           <t>C04 Pipe and cable bracket, wall hook</t>
         </is>
       </c>
-      <c r="B29" s="8" t="n"/>
-      <c r="C29" s="24" t="n"/>
-      <c r="D29" s="24" t="n"/>
-      <c r="E29" s="24" t="n"/>
-      <c r="F29" s="24" t="n"/>
-      <c r="G29" s="24" t="n"/>
-      <c r="I29" s="27" t="n"/>
-      <c r="J29" s="27" t="n"/>
-      <c r="K29" s="27" t="n"/>
-      <c r="L29" s="27" t="n"/>
-      <c r="M29" s="27" t="n"/>
-      <c r="N29" s="27" t="n"/>
-      <c r="O29" s="27" t="n"/>
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t>10 to 30</t>
+        </is>
+      </c>
+      <c r="C29" s="25" t="n"/>
+      <c r="D29" s="25" t="n"/>
+      <c r="E29" s="25" t="n"/>
+      <c r="F29" s="25" t="n"/>
+      <c r="G29" s="25" t="n"/>
+      <c r="I29" s="28" t="n"/>
+      <c r="J29" s="28" t="n"/>
+      <c r="K29" s="28" t="n"/>
+      <c r="L29" s="28" t="n"/>
+      <c r="M29" s="28" t="n"/>
+      <c r="N29" s="28" t="n"/>
+      <c r="O29" s="28" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="23" t="inlineStr">
@@ -1970,12 +2108,16 @@
           <t>C05 Handrail: straight, post, bend, end cap</t>
         </is>
       </c>
-      <c r="B30" s="8" t="n"/>
-      <c r="C30" s="24" t="n"/>
-      <c r="D30" s="24" t="n"/>
-      <c r="E30" s="24" t="n"/>
-      <c r="F30" s="24" t="n"/>
-      <c r="G30" s="24" t="n"/>
+      <c r="B30" s="24" t="inlineStr">
+        <is>
+          <t>100, 150, 200</t>
+        </is>
+      </c>
+      <c r="C30" s="25" t="n"/>
+      <c r="D30" s="25" t="n"/>
+      <c r="E30" s="25" t="n"/>
+      <c r="F30" s="25" t="n"/>
+      <c r="G30" s="25" t="n"/>
       <c r="I30" s="19" t="inlineStr">
         <is>
           <t>Week 8 · Props and debris</t>
@@ -1994,12 +2136,16 @@
           <t>C06 Gutter run and bracket</t>
         </is>
       </c>
-      <c r="B31" s="8" t="n"/>
-      <c r="C31" s="24" t="n"/>
-      <c r="D31" s="24" t="n"/>
-      <c r="E31" s="24" t="n"/>
-      <c r="F31" s="24" t="n"/>
-      <c r="G31" s="24" t="n"/>
+      <c r="B31" s="24" t="inlineStr">
+        <is>
+          <t>200, 400</t>
+        </is>
+      </c>
+      <c r="C31" s="25" t="n"/>
+      <c r="D31" s="25" t="n"/>
+      <c r="E31" s="25" t="n"/>
+      <c r="F31" s="25" t="n"/>
+      <c r="G31" s="25" t="n"/>
       <c r="I31" s="22" t="n">
         <v>46363</v>
       </c>
@@ -2028,7 +2174,11 @@
           <t>Kit D · Ground</t>
         </is>
       </c>
-      <c r="B32" s="29" t="n"/>
+      <c r="B32" s="31" t="inlineStr">
+        <is>
+          <t>Size (cm)</t>
+        </is>
+      </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
           <t>Blockout</t>
@@ -2054,37 +2204,37 @@
           <t>In UE5</t>
         </is>
       </c>
-      <c r="I32" s="25" t="inlineStr">
+      <c r="I32" s="26" t="inlineStr">
         <is>
           <t>P01 plywood, P02 planks, P03 offcuts</t>
         </is>
       </c>
-      <c r="J32" s="25" t="inlineStr">
+      <c r="J32" s="26" t="inlineStr">
         <is>
           <t>P04 bricks and P05 rubble piles</t>
         </is>
       </c>
-      <c r="K32" s="26" t="inlineStr">
+      <c r="K32" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="L32" s="26" t="inlineStr">
+      <c r="L32" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="M32" s="25" t="inlineStr">
+      <c r="M32" s="26" t="inlineStr">
         <is>
           <t>P06 pipes, P07 cable spline, P08 fallen gutter, P09 broken frame</t>
         </is>
       </c>
-      <c r="N32" s="25" t="inlineStr">
+      <c r="N32" s="26" t="inlineStr">
         <is>
           <t>P10 glass shards, P11 dead branches, P12 corrugated sheet, P15 litter, P16 paper</t>
         </is>
       </c>
-      <c r="O32" s="25" t="inlineStr">
+      <c r="O32" s="26" t="inlineStr">
         <is>
           <t>P17 junction box, P18 lamp bracket, then P3 props if time + Review 8</t>
         </is>
@@ -2098,48 +2248,58 @@
       <c r="E33" s="21" t="n"/>
       <c r="F33" s="21" t="n"/>
       <c r="G33" s="21" t="n"/>
-      <c r="I33" s="27" t="n"/>
-      <c r="J33" s="27" t="n"/>
-      <c r="K33" s="27" t="n"/>
-      <c r="L33" s="27" t="n"/>
-      <c r="M33" s="27" t="n"/>
-      <c r="N33" s="27" t="n"/>
-      <c r="O33" s="27" t="n"/>
+      <c r="I33" s="28" t="n"/>
+      <c r="J33" s="28" t="n"/>
+      <c r="K33" s="28" t="n"/>
+      <c r="L33" s="28" t="n"/>
+      <c r="M33" s="28" t="n"/>
+      <c r="N33" s="28" t="n"/>
+      <c r="O33" s="28" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="28" t="inlineStr">
+      <c r="A34" s="30" t="inlineStr">
         <is>
           <t>D01 Ground tile, setts under mud</t>
         </is>
       </c>
-      <c r="C34" s="33" t="n"/>
-      <c r="D34" s="33" t="n"/>
-      <c r="E34" s="33" t="n"/>
-      <c r="F34" s="33" t="n"/>
-      <c r="G34" s="33" t="n"/>
-      <c r="I34" s="29" t="inlineStr">
+      <c r="B34" s="29" t="inlineStr">
+        <is>
+          <t>400 x 400</t>
+        </is>
+      </c>
+      <c r="C34" s="35" t="n"/>
+      <c r="D34" s="35" t="n"/>
+      <c r="E34" s="35" t="n"/>
+      <c r="F34" s="35" t="n"/>
+      <c r="G34" s="35" t="n"/>
+      <c r="I34" s="31" t="inlineStr">
         <is>
           <t>Week 9 · Foliage</t>
         </is>
       </c>
-      <c r="J34" s="29" t="n"/>
-      <c r="K34" s="29" t="n"/>
-      <c r="L34" s="29" t="n"/>
-      <c r="M34" s="29" t="n"/>
-      <c r="N34" s="29" t="n"/>
-      <c r="O34" s="29" t="n"/>
+      <c r="J34" s="31" t="n"/>
+      <c r="K34" s="31" t="n"/>
+      <c r="L34" s="31" t="n"/>
+      <c r="M34" s="31" t="n"/>
+      <c r="N34" s="31" t="n"/>
+      <c r="O34" s="31" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="28" t="inlineStr">
+      <c r="A35" s="30" t="inlineStr">
         <is>
           <t>D02 Kerb / wall-base strip</t>
         </is>
       </c>
-      <c r="C35" s="33" t="n"/>
-      <c r="D35" s="33" t="n"/>
-      <c r="E35" s="33" t="n"/>
-      <c r="F35" s="33" t="n"/>
-      <c r="G35" s="33" t="n"/>
+      <c r="B35" s="29" t="inlineStr">
+        <is>
+          <t>400 long</t>
+        </is>
+      </c>
+      <c r="C35" s="35" t="n"/>
+      <c r="D35" s="35" t="n"/>
+      <c r="E35" s="35" t="n"/>
+      <c r="F35" s="35" t="n"/>
+      <c r="G35" s="35" t="n"/>
       <c r="I35" s="22" t="n">
         <v>46370</v>
       </c>
@@ -2163,47 +2323,52 @@
       </c>
     </row>
     <row r="36" ht="58" customHeight="1" s="17">
-      <c r="A36" s="28" t="inlineStr">
+      <c r="A36" s="30" t="inlineStr">
         <is>
           <t>D03 Drain grate and channel</t>
         </is>
       </c>
-      <c r="C36" s="33" t="n"/>
-      <c r="D36" s="33" t="n"/>
-      <c r="E36" s="33" t="n"/>
-      <c r="F36" s="33" t="n"/>
-      <c r="G36" s="33" t="n"/>
-      <c r="I36" s="25" t="inlineStr">
+      <c r="B36" s="29" t="inlineStr">
+        <is>
+          <t>100 x 30</t>
+        </is>
+      </c>
+      <c r="C36" s="35" t="n"/>
+      <c r="D36" s="35" t="n"/>
+      <c r="E36" s="35" t="n"/>
+      <c r="F36" s="35" t="n"/>
+      <c r="G36" s="35" t="n"/>
+      <c r="I36" s="26" t="inlineStr">
         <is>
           <t>Model leaves</t>
         </is>
       </c>
-      <c r="J36" s="25" t="inlineStr">
+      <c r="J36" s="26" t="inlineStr">
         <is>
           <t>F01 ivy cards and vine splines</t>
         </is>
       </c>
-      <c r="K36" s="26" t="inlineStr">
+      <c r="K36" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="L36" s="26" t="inlineStr">
+      <c r="L36" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="M36" s="25" t="inlineStr">
+      <c r="M36" s="26" t="inlineStr">
         <is>
           <t>F02 moss clumps, F03 grass and weeds, F05 dead leaves</t>
         </is>
       </c>
-      <c r="N36" s="25" t="inlineStr">
+      <c r="N36" s="26" t="inlineStr">
         <is>
           <t>F04 buddleia, F06 brambles, F07 saplings</t>
         </is>
       </c>
-      <c r="O36" s="25" t="inlineStr">
+      <c r="O36" s="26" t="inlineStr">
         <is>
           <t>F08 background trees and the H5 far opening mass + Review 9</t>
         </is>
@@ -2215,19 +2380,23 @@
           <t>D04 Rubble edge strip (ground meets wall)</t>
         </is>
       </c>
-      <c r="B37" s="10" t="n"/>
-      <c r="C37" s="33" t="n"/>
-      <c r="D37" s="33" t="n"/>
-      <c r="E37" s="33" t="n"/>
-      <c r="F37" s="33" t="n"/>
-      <c r="G37" s="33" t="n"/>
-      <c r="I37" s="34" t="n"/>
-      <c r="J37" s="34" t="n"/>
-      <c r="K37" s="34" t="n"/>
-      <c r="L37" s="34" t="n"/>
-      <c r="M37" s="34" t="n"/>
-      <c r="N37" s="34" t="n"/>
-      <c r="O37" s="34" t="n"/>
+      <c r="B37" s="29" t="inlineStr">
+        <is>
+          <t>400 long</t>
+        </is>
+      </c>
+      <c r="C37" s="35" t="n"/>
+      <c r="D37" s="35" t="n"/>
+      <c r="E37" s="35" t="n"/>
+      <c r="F37" s="35" t="n"/>
+      <c r="G37" s="35" t="n"/>
+      <c r="I37" s="36" t="n"/>
+      <c r="J37" s="36" t="n"/>
+      <c r="K37" s="36" t="n"/>
+      <c r="L37" s="36" t="n"/>
+      <c r="M37" s="36" t="n"/>
+      <c r="N37" s="36" t="n"/>
+      <c r="O37" s="36" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="23" t="inlineStr">
@@ -2235,23 +2404,27 @@
           <t>D05 Broken ground patch (exposed setts)</t>
         </is>
       </c>
-      <c r="B38" s="10" t="n"/>
-      <c r="C38" s="33" t="n"/>
-      <c r="D38" s="33" t="n"/>
-      <c r="E38" s="33" t="n"/>
-      <c r="F38" s="33" t="n"/>
-      <c r="G38" s="33" t="n"/>
-      <c r="I38" s="29" t="inlineStr">
+      <c r="B38" s="29" t="inlineStr">
+        <is>
+          <t>200 x 200</t>
+        </is>
+      </c>
+      <c r="C38" s="35" t="n"/>
+      <c r="D38" s="35" t="n"/>
+      <c r="E38" s="35" t="n"/>
+      <c r="F38" s="35" t="n"/>
+      <c r="G38" s="35" t="n"/>
+      <c r="I38" s="31" t="inlineStr">
         <is>
           <t>Week 10 · Decals and vertex paint</t>
         </is>
       </c>
-      <c r="J38" s="29" t="n"/>
-      <c r="K38" s="29" t="n"/>
-      <c r="L38" s="29" t="n"/>
-      <c r="M38" s="29" t="n"/>
-      <c r="N38" s="29" t="n"/>
-      <c r="O38" s="29" t="n"/>
+      <c r="J38" s="31" t="n"/>
+      <c r="K38" s="31" t="n"/>
+      <c r="L38" s="31" t="n"/>
+      <c r="M38" s="31" t="n"/>
+      <c r="N38" s="31" t="n"/>
+      <c r="O38" s="31" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="23" t="inlineStr">
@@ -2259,12 +2432,16 @@
           <t>D06 Puddle insert (shallow depression)</t>
         </is>
       </c>
-      <c r="B39" s="10" t="n"/>
-      <c r="C39" s="33" t="n"/>
-      <c r="D39" s="33" t="n"/>
-      <c r="E39" s="33" t="n"/>
-      <c r="F39" s="33" t="n"/>
-      <c r="G39" s="33" t="n"/>
+      <c r="B39" s="29" t="inlineStr">
+        <is>
+          <t>150 x 100</t>
+        </is>
+      </c>
+      <c r="C39" s="35" t="n"/>
+      <c r="D39" s="35" t="n"/>
+      <c r="E39" s="35" t="n"/>
+      <c r="F39" s="35" t="n"/>
+      <c r="G39" s="35" t="n"/>
       <c r="I39" s="22" t="n">
         <v>46377</v>
       </c>
@@ -2288,123 +2465,137 @@
       </c>
     </row>
     <row r="40" ht="58" customHeight="1" s="17">
-      <c r="A40" s="28" t="inlineStr">
+      <c r="A40" s="30" t="inlineStr">
         <is>
           <t>D07 Wall-base dirt pile</t>
         </is>
       </c>
-      <c r="C40" s="33" t="n"/>
-      <c r="D40" s="33" t="n"/>
-      <c r="E40" s="33" t="n"/>
-      <c r="F40" s="33" t="n"/>
-      <c r="G40" s="33" t="n"/>
-      <c r="I40" s="25" t="inlineStr">
+      <c r="B40" s="29" t="inlineStr">
+        <is>
+          <t>200 long</t>
+        </is>
+      </c>
+      <c r="C40" s="35" t="n"/>
+      <c r="D40" s="35" t="n"/>
+      <c r="E40" s="35" t="n"/>
+      <c r="F40" s="35" t="n"/>
+      <c r="G40" s="35" t="n"/>
+      <c r="I40" s="26" t="inlineStr">
         <is>
           <t>Build decals X01 to X04 and M_Master_Decal</t>
         </is>
       </c>
-      <c r="J40" s="25" t="inlineStr">
+      <c r="J40" s="26" t="inlineStr">
         <is>
           <t>Build decals X05 to X08</t>
         </is>
       </c>
-      <c r="K40" s="26" t="inlineStr">
+      <c r="K40" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="L40" s="26" t="inlineStr">
+      <c r="L40" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="M40" s="32" t="inlineStr">
+      <c r="M40" s="34" t="inlineStr">
         <is>
           <t>Buffer (Christmas)</t>
         </is>
       </c>
-      <c r="N40" s="25" t="inlineStr">
+      <c r="N40" s="26" t="inlineStr">
         <is>
           <t>Vertex paint both facades</t>
         </is>
       </c>
-      <c r="O40" s="25" t="inlineStr">
+      <c r="O40" s="26" t="inlineStr">
         <is>
           <t>Place decals + Review 10</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="29" t="inlineStr">
+      <c r="A41" s="31" t="inlineStr">
         <is>
           <t>Hero features</t>
         </is>
       </c>
-      <c r="B41" s="29" t="n"/>
-      <c r="C41" s="29" t="inlineStr">
+      <c r="B41" s="31" t="inlineStr">
+        <is>
+          <t>Size (cm)</t>
+        </is>
+      </c>
+      <c r="C41" s="31" t="inlineStr">
         <is>
           <t>Blockout</t>
         </is>
       </c>
-      <c r="D41" s="29" t="inlineStr">
+      <c r="D41" s="31" t="inlineStr">
         <is>
           <t>Highpoly</t>
         </is>
       </c>
-      <c r="E41" s="29" t="inlineStr">
+      <c r="E41" s="31" t="inlineStr">
         <is>
           <t>Lowpoly</t>
         </is>
       </c>
-      <c r="F41" s="29" t="inlineStr">
+      <c r="F41" s="31" t="inlineStr">
         <is>
           <t>Texture</t>
         </is>
       </c>
-      <c r="G41" s="29" t="inlineStr">
+      <c r="G41" s="31" t="inlineStr">
         <is>
           <t>In UE5</t>
         </is>
       </c>
-      <c r="I41" s="34" t="n"/>
-      <c r="J41" s="34" t="n"/>
-      <c r="K41" s="34" t="n"/>
-      <c r="L41" s="34" t="n"/>
-      <c r="M41" s="34" t="n"/>
-      <c r="N41" s="34" t="n"/>
-      <c r="O41" s="34" t="n"/>
+      <c r="I41" s="36" t="n"/>
+      <c r="J41" s="36" t="n"/>
+      <c r="K41" s="36" t="n"/>
+      <c r="L41" s="36" t="n"/>
+      <c r="M41" s="36" t="n"/>
+      <c r="N41" s="36" t="n"/>
+      <c r="O41" s="36" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="30" t="n"/>
-      <c r="B42" s="30" t="n"/>
-      <c r="C42" s="30" t="n"/>
-      <c r="D42" s="30" t="n"/>
-      <c r="E42" s="30" t="n"/>
-      <c r="F42" s="30" t="n"/>
-      <c r="G42" s="30" t="n"/>
-      <c r="I42" s="29" t="inlineStr">
+      <c r="A42" s="32" t="n"/>
+      <c r="B42" s="32" t="n"/>
+      <c r="C42" s="32" t="n"/>
+      <c r="D42" s="32" t="n"/>
+      <c r="E42" s="32" t="n"/>
+      <c r="F42" s="32" t="n"/>
+      <c r="G42" s="32" t="n"/>
+      <c r="I42" s="31" t="inlineStr">
         <is>
           <t>Week 11 · Set dressing</t>
         </is>
       </c>
-      <c r="J42" s="29" t="n"/>
-      <c r="K42" s="29" t="n"/>
-      <c r="L42" s="29" t="n"/>
-      <c r="M42" s="29" t="n"/>
-      <c r="N42" s="29" t="n"/>
-      <c r="O42" s="29" t="n"/>
+      <c r="J42" s="31" t="n"/>
+      <c r="K42" s="31" t="n"/>
+      <c r="L42" s="31" t="n"/>
+      <c r="M42" s="31" t="n"/>
+      <c r="N42" s="31" t="n"/>
+      <c r="O42" s="31" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="28" t="inlineStr">
+      <c r="A43" s="30" t="inlineStr">
         <is>
           <t>H1 Two-tier skybridge</t>
         </is>
       </c>
-      <c r="C43" s="33" t="n"/>
-      <c r="D43" s="33" t="n"/>
-      <c r="E43" s="33" t="n"/>
-      <c r="F43" s="33" t="n"/>
-      <c r="G43" s="33" t="n"/>
+      <c r="B43" s="29" t="inlineStr">
+        <is>
+          <t>500 span x 340 h x 250 d</t>
+        </is>
+      </c>
+      <c r="C43" s="35" t="n"/>
+      <c r="D43" s="35" t="n"/>
+      <c r="E43" s="35" t="n"/>
+      <c r="F43" s="35" t="n"/>
+      <c r="G43" s="35" t="n"/>
       <c r="I43" s="22" t="n">
         <v>46384</v>
       </c>
@@ -2428,105 +2619,117 @@
       </c>
     </row>
     <row r="44" ht="58" customHeight="1" s="17">
-      <c r="A44" s="28" t="inlineStr">
+      <c r="A44" s="30" t="inlineStr">
         <is>
           <t>H2 Chimney stack and red end building</t>
         </is>
       </c>
-      <c r="C44" s="33" t="n"/>
-      <c r="D44" s="33" t="n"/>
-      <c r="E44" s="33" t="n"/>
-      <c r="F44" s="33" t="n"/>
-      <c r="G44" s="33" t="n"/>
-      <c r="I44" s="25" t="inlineStr">
+      <c r="B44" s="29" t="inlineStr">
+        <is>
+          <t>180 x 2800 h x 180</t>
+        </is>
+      </c>
+      <c r="C44" s="35" t="n"/>
+      <c r="D44" s="35" t="n"/>
+      <c r="E44" s="35" t="n"/>
+      <c r="F44" s="35" t="n"/>
+      <c r="G44" s="35" t="n"/>
+      <c r="I44" s="26" t="inlineStr">
         <is>
           <t>Ground dressing</t>
         </is>
       </c>
-      <c r="J44" s="25" t="inlineStr">
+      <c r="J44" s="26" t="inlineStr">
         <is>
           <t>Place P1 props in Camera 1 for composition</t>
         </is>
       </c>
-      <c r="K44" s="26" t="inlineStr">
+      <c r="K44" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="L44" s="26" t="inlineStr">
+      <c r="L44" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="M44" s="32" t="inlineStr">
+      <c r="M44" s="34" t="inlineStr">
         <is>
           <t>Buffer (New Year's Day)</t>
         </is>
       </c>
-      <c r="N44" s="25" t="inlineStr">
+      <c r="N44" s="26" t="inlineStr">
         <is>
           <t>Foliage placement + Review 11</t>
         </is>
       </c>
-      <c r="O44" s="32" t="inlineStr">
+      <c r="O44" s="34" t="inlineStr">
         <is>
           <t>Buffer</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="28" t="inlineStr">
+      <c r="A45" s="30" t="inlineStr">
         <is>
           <t>H3 Basement light well with green handrail</t>
         </is>
       </c>
-      <c r="C45" s="33" t="n"/>
-      <c r="D45" s="33" t="n"/>
-      <c r="E45" s="33" t="n"/>
-      <c r="F45" s="33" t="n"/>
-      <c r="G45" s="33" t="n"/>
-      <c r="I45" s="34" t="n"/>
-      <c r="J45" s="34" t="n"/>
-      <c r="K45" s="34" t="n"/>
-      <c r="L45" s="34" t="n"/>
-      <c r="M45" s="34" t="n"/>
-      <c r="N45" s="34" t="n"/>
-      <c r="O45" s="34" t="n"/>
+      <c r="B45" s="29" t="inlineStr">
+        <is>
+          <t>120 x 200 drop x 380</t>
+        </is>
+      </c>
+      <c r="C45" s="35" t="n"/>
+      <c r="D45" s="35" t="n"/>
+      <c r="E45" s="35" t="n"/>
+      <c r="F45" s="35" t="n"/>
+      <c r="G45" s="35" t="n"/>
+      <c r="I45" s="36" t="n"/>
+      <c r="J45" s="36" t="n"/>
+      <c r="K45" s="36" t="n"/>
+      <c r="L45" s="36" t="n"/>
+      <c r="M45" s="36" t="n"/>
+      <c r="N45" s="36" t="n"/>
+      <c r="O45" s="36" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="28" t="inlineStr">
+      <c r="A46" s="30" t="inlineStr">
         <is>
           <t>H4 Cascading ivy and wall growth</t>
         </is>
       </c>
-      <c r="C46" s="33" t="n"/>
-      <c r="D46" s="33" t="n"/>
-      <c r="E46" s="33" t="n"/>
-      <c r="F46" s="33" t="n"/>
-      <c r="G46" s="33" t="n"/>
-      <c r="I46" s="29" t="inlineStr">
+      <c r="B46" s="29" t="n"/>
+      <c r="C46" s="35" t="n"/>
+      <c r="D46" s="35" t="n"/>
+      <c r="E46" s="35" t="n"/>
+      <c r="F46" s="35" t="n"/>
+      <c r="G46" s="35" t="n"/>
+      <c r="I46" s="31" t="inlineStr">
         <is>
           <t>Week 12 · Dressing for alternate angles</t>
         </is>
       </c>
-      <c r="J46" s="29" t="n"/>
-      <c r="K46" s="29" t="n"/>
-      <c r="L46" s="29" t="n"/>
-      <c r="M46" s="29" t="n"/>
-      <c r="N46" s="29" t="n"/>
-      <c r="O46" s="29" t="n"/>
+      <c r="J46" s="31" t="n"/>
+      <c r="K46" s="31" t="n"/>
+      <c r="L46" s="31" t="n"/>
+      <c r="M46" s="31" t="n"/>
+      <c r="N46" s="31" t="n"/>
+      <c r="O46" s="31" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="28" t="inlineStr">
+      <c r="A47" s="30" t="inlineStr">
         <is>
           <t>H5 Overgrown far opening</t>
         </is>
       </c>
-      <c r="C47" s="33" t="n"/>
-      <c r="D47" s="33" t="n"/>
-      <c r="E47" s="33" t="n"/>
-      <c r="F47" s="33" t="n"/>
-      <c r="G47" s="33" t="n"/>
+      <c r="B47" s="29" t="n"/>
+      <c r="C47" s="35" t="n"/>
+      <c r="D47" s="35" t="n"/>
+      <c r="E47" s="35" t="n"/>
+      <c r="F47" s="35" t="n"/>
+      <c r="G47" s="35" t="n"/>
       <c r="I47" s="22" t="n">
         <v>46391</v>
       </c>
@@ -2550,123 +2753,137 @@
       </c>
     </row>
     <row r="48" ht="58" customHeight="1" s="17">
-      <c r="A48" s="28" t="inlineStr">
+      <c r="A48" s="30" t="inlineStr">
         <is>
           <t>H6 Rusted arched loading doors</t>
         </is>
       </c>
-      <c r="C48" s="33" t="n"/>
-      <c r="D48" s="33" t="n"/>
-      <c r="E48" s="33" t="n"/>
-      <c r="F48" s="33" t="n"/>
-      <c r="G48" s="33" t="n"/>
-      <c r="I48" s="25" t="inlineStr">
+      <c r="B48" s="29" t="inlineStr">
+        <is>
+          <t>240 x 320</t>
+        </is>
+      </c>
+      <c r="C48" s="35" t="n"/>
+      <c r="D48" s="35" t="n"/>
+      <c r="E48" s="35" t="n"/>
+      <c r="F48" s="35" t="n"/>
+      <c r="G48" s="35" t="n"/>
+      <c r="I48" s="26" t="inlineStr">
         <is>
           <t>Dress the alternate cameras with P2 props, glass, litter, paper</t>
         </is>
       </c>
-      <c r="J48" s="25" t="inlineStr">
+      <c r="J48" s="26" t="inlineStr">
         <is>
           <t>Puddles and wetness</t>
         </is>
       </c>
-      <c r="K48" s="26" t="inlineStr">
+      <c r="K48" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="L48" s="26" t="inlineStr">
+      <c r="L48" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="M48" s="32" t="inlineStr">
+      <c r="M48" s="34" t="inlineStr">
         <is>
           <t>Buffer</t>
         </is>
       </c>
-      <c r="N48" s="25" t="inlineStr">
+      <c r="N48" s="26" t="inlineStr">
         <is>
           <t>Full walkthrough + Review 12</t>
         </is>
       </c>
-      <c r="O48" s="32" t="inlineStr">
+      <c r="O48" s="34" t="inlineStr">
         <is>
           <t>Buffer</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="28" t="inlineStr">
+      <c r="A49" s="30" t="inlineStr">
         <is>
           <t>H7 Broken industrial glazing</t>
         </is>
       </c>
-      <c r="C49" s="33" t="n"/>
-      <c r="D49" s="33" t="n"/>
-      <c r="E49" s="33" t="n"/>
-      <c r="F49" s="33" t="n"/>
-      <c r="G49" s="33" t="n"/>
-      <c r="I49" s="34" t="n"/>
-      <c r="J49" s="34" t="n"/>
-      <c r="K49" s="34" t="n"/>
-      <c r="L49" s="34" t="n"/>
-      <c r="M49" s="34" t="n"/>
-      <c r="N49" s="34" t="n"/>
-      <c r="O49" s="34" t="n"/>
+      <c r="B49" s="29" t="inlineStr">
+        <is>
+          <t>140 x 220</t>
+        </is>
+      </c>
+      <c r="C49" s="35" t="n"/>
+      <c r="D49" s="35" t="n"/>
+      <c r="E49" s="35" t="n"/>
+      <c r="F49" s="35" t="n"/>
+      <c r="G49" s="35" t="n"/>
+      <c r="I49" s="36" t="n"/>
+      <c r="J49" s="36" t="n"/>
+      <c r="K49" s="36" t="n"/>
+      <c r="L49" s="36" t="n"/>
+      <c r="M49" s="36" t="n"/>
+      <c r="N49" s="36" t="n"/>
+      <c r="O49" s="36" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="29" t="inlineStr">
+      <c r="A50" s="31" t="inlineStr">
         <is>
           <t>Props</t>
         </is>
       </c>
-      <c r="B50" s="29" t="n"/>
-      <c r="C50" s="29" t="inlineStr">
+      <c r="B50" s="31" t="inlineStr">
+        <is>
+          <t>Size (cm)</t>
+        </is>
+      </c>
+      <c r="C50" s="31" t="inlineStr">
         <is>
           <t>Blockout</t>
         </is>
       </c>
-      <c r="D50" s="29" t="inlineStr">
+      <c r="D50" s="31" t="inlineStr">
         <is>
           <t>Highpoly</t>
         </is>
       </c>
-      <c r="E50" s="29" t="inlineStr">
+      <c r="E50" s="31" t="inlineStr">
         <is>
           <t>Lowpoly</t>
         </is>
       </c>
-      <c r="F50" s="29" t="inlineStr">
+      <c r="F50" s="31" t="inlineStr">
         <is>
           <t>Texture</t>
         </is>
       </c>
-      <c r="G50" s="29" t="inlineStr">
+      <c r="G50" s="31" t="inlineStr">
         <is>
           <t>In UE5</t>
         </is>
       </c>
-      <c r="I50" s="29" t="inlineStr">
+      <c r="I50" s="31" t="inlineStr">
         <is>
           <t>Week 13 · Lighting and atmosphere</t>
         </is>
       </c>
-      <c r="J50" s="29" t="n"/>
-      <c r="K50" s="29" t="n"/>
-      <c r="L50" s="29" t="n"/>
-      <c r="M50" s="29" t="n"/>
-      <c r="N50" s="29" t="n"/>
-      <c r="O50" s="29" t="n"/>
+      <c r="J50" s="31" t="n"/>
+      <c r="K50" s="31" t="n"/>
+      <c r="L50" s="31" t="n"/>
+      <c r="M50" s="31" t="n"/>
+      <c r="N50" s="31" t="n"/>
+      <c r="O50" s="31" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="30" t="n"/>
-      <c r="B51" s="30" t="n"/>
-      <c r="C51" s="30" t="n"/>
-      <c r="D51" s="30" t="n"/>
-      <c r="E51" s="30" t="n"/>
-      <c r="F51" s="30" t="n"/>
-      <c r="G51" s="30" t="n"/>
+      <c r="A51" s="32" t="n"/>
+      <c r="B51" s="32" t="n"/>
+      <c r="C51" s="32" t="n"/>
+      <c r="D51" s="32" t="n"/>
+      <c r="E51" s="32" t="n"/>
+      <c r="F51" s="32" t="n"/>
+      <c r="G51" s="32" t="n"/>
       <c r="I51" s="22" t="n">
         <v>46398</v>
       </c>
@@ -2690,105 +2907,125 @@
       </c>
     </row>
     <row r="52" ht="58" customHeight="1" s="17">
-      <c r="A52" s="28" t="inlineStr">
+      <c r="A52" s="30" t="inlineStr">
         <is>
           <t>P01 Plywood sheet, warped and delaminating</t>
         </is>
       </c>
-      <c r="C52" s="33" t="n"/>
-      <c r="D52" s="33" t="n"/>
-      <c r="E52" s="33" t="n"/>
-      <c r="F52" s="33" t="n"/>
-      <c r="G52" s="33" t="n"/>
-      <c r="I52" s="25" t="inlineStr">
+      <c r="B52" s="29" t="inlineStr">
+        <is>
+          <t>122 x 244</t>
+        </is>
+      </c>
+      <c r="C52" s="35" t="n"/>
+      <c r="D52" s="35" t="n"/>
+      <c r="E52" s="35" t="n"/>
+      <c r="F52" s="35" t="n"/>
+      <c r="G52" s="35" t="n"/>
+      <c r="I52" s="26" t="inlineStr">
         <is>
           <t>Overcast sky</t>
         </is>
       </c>
-      <c r="J52" s="25" t="inlineStr">
+      <c r="J52" s="26" t="inlineStr">
         <is>
           <t>Height fog and volumetrics</t>
         </is>
       </c>
-      <c r="K52" s="26" t="inlineStr">
+      <c r="K52" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="L52" s="26" t="inlineStr">
+      <c r="L52" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="M52" s="25" t="inlineStr">
+      <c r="M52" s="26" t="inlineStr">
         <is>
           <t>Post process</t>
         </is>
       </c>
-      <c r="N52" s="25" t="inlineStr">
+      <c r="N52" s="26" t="inlineStr">
         <is>
           <t>Light the alternate cameras</t>
         </is>
       </c>
-      <c r="O52" s="25" t="inlineStr">
+      <c r="O52" s="26" t="inlineStr">
         <is>
           <t>Review 13</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="28" t="inlineStr">
+      <c r="A53" s="30" t="inlineStr">
         <is>
           <t>P02 Timber planks, 4 variants</t>
         </is>
       </c>
-      <c r="C53" s="33" t="n"/>
-      <c r="D53" s="33" t="n"/>
-      <c r="E53" s="33" t="n"/>
-      <c r="F53" s="33" t="n"/>
-      <c r="G53" s="33" t="n"/>
-      <c r="I53" s="34" t="n"/>
-      <c r="J53" s="34" t="n"/>
-      <c r="K53" s="34" t="n"/>
-      <c r="L53" s="34" t="n"/>
-      <c r="M53" s="34" t="n"/>
-      <c r="N53" s="34" t="n"/>
-      <c r="O53" s="34" t="n"/>
+      <c r="B53" s="29" t="inlineStr">
+        <is>
+          <t>15 x 240</t>
+        </is>
+      </c>
+      <c r="C53" s="35" t="n"/>
+      <c r="D53" s="35" t="n"/>
+      <c r="E53" s="35" t="n"/>
+      <c r="F53" s="35" t="n"/>
+      <c r="G53" s="35" t="n"/>
+      <c r="I53" s="36" t="n"/>
+      <c r="J53" s="36" t="n"/>
+      <c r="K53" s="36" t="n"/>
+      <c r="L53" s="36" t="n"/>
+      <c r="M53" s="36" t="n"/>
+      <c r="N53" s="36" t="n"/>
+      <c r="O53" s="36" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="28" t="inlineStr">
+      <c r="A54" s="30" t="inlineStr">
         <is>
           <t>P03 Broken timber offcuts, 6 variants</t>
         </is>
       </c>
-      <c r="C54" s="33" t="n"/>
-      <c r="D54" s="33" t="n"/>
-      <c r="E54" s="33" t="n"/>
-      <c r="F54" s="33" t="n"/>
-      <c r="G54" s="33" t="n"/>
-      <c r="I54" s="29" t="inlineStr">
+      <c r="B54" s="29" t="inlineStr">
+        <is>
+          <t>10 to 60</t>
+        </is>
+      </c>
+      <c r="C54" s="35" t="n"/>
+      <c r="D54" s="35" t="n"/>
+      <c r="E54" s="35" t="n"/>
+      <c r="F54" s="35" t="n"/>
+      <c r="G54" s="35" t="n"/>
+      <c r="I54" s="31" t="inlineStr">
         <is>
           <t>Week 14 · Polish and optimization</t>
         </is>
       </c>
-      <c r="J54" s="29" t="n"/>
-      <c r="K54" s="29" t="n"/>
-      <c r="L54" s="29" t="n"/>
-      <c r="M54" s="29" t="n"/>
-      <c r="N54" s="29" t="n"/>
-      <c r="O54" s="29" t="n"/>
+      <c r="J54" s="31" t="n"/>
+      <c r="K54" s="31" t="n"/>
+      <c r="L54" s="31" t="n"/>
+      <c r="M54" s="31" t="n"/>
+      <c r="N54" s="31" t="n"/>
+      <c r="O54" s="31" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="28" t="inlineStr">
+      <c r="A55" s="30" t="inlineStr">
         <is>
           <t>P04 Loose bricks and half bricks, 6 variants</t>
         </is>
       </c>
-      <c r="C55" s="33" t="n"/>
-      <c r="D55" s="33" t="n"/>
-      <c r="E55" s="33" t="n"/>
-      <c r="F55" s="33" t="n"/>
-      <c r="G55" s="33" t="n"/>
+      <c r="B55" s="29" t="inlineStr">
+        <is>
+          <t>23 x 11</t>
+        </is>
+      </c>
+      <c r="C55" s="35" t="n"/>
+      <c r="D55" s="35" t="n"/>
+      <c r="E55" s="35" t="n"/>
+      <c r="F55" s="35" t="n"/>
+      <c r="G55" s="35" t="n"/>
       <c r="I55" s="22" t="n">
         <v>46405</v>
       </c>
@@ -2812,105 +3049,125 @@
       </c>
     </row>
     <row r="56" ht="58" customHeight="1" s="17">
-      <c r="A56" s="28" t="inlineStr">
+      <c r="A56" s="30" t="inlineStr">
         <is>
           <t>P05 Rubble pile cluster, 3 variants</t>
         </is>
       </c>
-      <c r="C56" s="33" t="n"/>
-      <c r="D56" s="33" t="n"/>
-      <c r="E56" s="33" t="n"/>
-      <c r="F56" s="33" t="n"/>
-      <c r="G56" s="33" t="n"/>
-      <c r="I56" s="25" t="inlineStr">
+      <c r="B56" s="29" t="inlineStr">
+        <is>
+          <t>100 to 200</t>
+        </is>
+      </c>
+      <c r="C56" s="35" t="n"/>
+      <c r="D56" s="35" t="n"/>
+      <c r="E56" s="35" t="n"/>
+      <c r="F56" s="35" t="n"/>
+      <c r="G56" s="35" t="n"/>
+      <c r="I56" s="26" t="inlineStr">
         <is>
           <t>Apply critique notes</t>
         </is>
       </c>
-      <c r="J56" s="25" t="inlineStr">
+      <c r="J56" s="26" t="inlineStr">
         <is>
           <t>Material polish</t>
         </is>
       </c>
-      <c r="K56" s="26" t="inlineStr">
+      <c r="K56" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="L56" s="26" t="inlineStr">
+      <c r="L56" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="M56" s="25" t="inlineStr">
+      <c r="M56" s="26" t="inlineStr">
         <is>
           <t>Optimization</t>
         </is>
       </c>
-      <c r="N56" s="25" t="inlineStr">
+      <c r="N56" s="26" t="inlineStr">
         <is>
           <t>Audit texel density, wireframes, naming</t>
         </is>
       </c>
-      <c r="O56" s="25" t="inlineStr">
+      <c r="O56" s="26" t="inlineStr">
         <is>
           <t>Final polish in Camera 1 + Review 14</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="28" t="inlineStr">
+      <c r="A57" s="30" t="inlineStr">
         <is>
           <t>P06 Rusted pipe lengths, 3 variants</t>
         </is>
       </c>
-      <c r="C57" s="33" t="n"/>
-      <c r="D57" s="33" t="n"/>
-      <c r="E57" s="33" t="n"/>
-      <c r="F57" s="33" t="n"/>
-      <c r="G57" s="33" t="n"/>
-      <c r="I57" s="34" t="n"/>
-      <c r="J57" s="34" t="n"/>
-      <c r="K57" s="34" t="n"/>
-      <c r="L57" s="34" t="n"/>
-      <c r="M57" s="34" t="n"/>
-      <c r="N57" s="34" t="n"/>
-      <c r="O57" s="34" t="n"/>
+      <c r="B57" s="29" t="inlineStr">
+        <is>
+          <t>100 to 300</t>
+        </is>
+      </c>
+      <c r="C57" s="35" t="n"/>
+      <c r="D57" s="35" t="n"/>
+      <c r="E57" s="35" t="n"/>
+      <c r="F57" s="35" t="n"/>
+      <c r="G57" s="35" t="n"/>
+      <c r="I57" s="36" t="n"/>
+      <c r="J57" s="36" t="n"/>
+      <c r="K57" s="36" t="n"/>
+      <c r="L57" s="36" t="n"/>
+      <c r="M57" s="36" t="n"/>
+      <c r="N57" s="36" t="n"/>
+      <c r="O57" s="36" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="28" t="inlineStr">
+      <c r="A58" s="30" t="inlineStr">
         <is>
           <t>P07 Hanging and loose cables, spline</t>
         </is>
       </c>
-      <c r="C58" s="33" t="n"/>
-      <c r="D58" s="33" t="n"/>
-      <c r="E58" s="33" t="n"/>
-      <c r="F58" s="33" t="n"/>
-      <c r="G58" s="33" t="n"/>
-      <c r="I58" s="29" t="inlineStr">
+      <c r="B58" s="29" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="C58" s="35" t="n"/>
+      <c r="D58" s="35" t="n"/>
+      <c r="E58" s="35" t="n"/>
+      <c r="F58" s="35" t="n"/>
+      <c r="G58" s="35" t="n"/>
+      <c r="I58" s="31" t="inlineStr">
         <is>
           <t>Week 15 · Final renders</t>
         </is>
       </c>
-      <c r="J58" s="29" t="n"/>
-      <c r="K58" s="29" t="n"/>
-      <c r="L58" s="29" t="n"/>
-      <c r="M58" s="29" t="n"/>
-      <c r="N58" s="29" t="n"/>
-      <c r="O58" s="29" t="n"/>
+      <c r="J58" s="31" t="n"/>
+      <c r="K58" s="31" t="n"/>
+      <c r="L58" s="31" t="n"/>
+      <c r="M58" s="31" t="n"/>
+      <c r="N58" s="31" t="n"/>
+      <c r="O58" s="31" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="28" t="inlineStr">
+      <c r="A59" s="30" t="inlineStr">
         <is>
           <t>P08 Fallen gutter section</t>
         </is>
       </c>
-      <c r="C59" s="33" t="n"/>
-      <c r="D59" s="33" t="n"/>
-      <c r="E59" s="33" t="n"/>
-      <c r="F59" s="33" t="n"/>
-      <c r="G59" s="33" t="n"/>
+      <c r="B59" s="29" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C59" s="35" t="n"/>
+      <c r="D59" s="35" t="n"/>
+      <c r="E59" s="35" t="n"/>
+      <c r="F59" s="35" t="n"/>
+      <c r="G59" s="35" t="n"/>
       <c r="I59" s="22" t="n">
         <v>46412</v>
       </c>
@@ -2934,793 +3191,963 @@
       </c>
     </row>
     <row r="60" ht="58" customHeight="1" s="17">
-      <c r="A60" s="28" t="inlineStr">
+      <c r="A60" s="30" t="inlineStr">
         <is>
           <t>P09 Broken window frame on ground</t>
         </is>
       </c>
-      <c r="C60" s="33" t="n"/>
-      <c r="D60" s="33" t="n"/>
-      <c r="E60" s="33" t="n"/>
-      <c r="F60" s="33" t="n"/>
-      <c r="G60" s="33" t="n"/>
-      <c r="I60" s="25" t="inlineStr">
+      <c r="B60" s="29" t="inlineStr">
+        <is>
+          <t>140 x 220</t>
+        </is>
+      </c>
+      <c r="C60" s="35" t="n"/>
+      <c r="D60" s="35" t="n"/>
+      <c r="E60" s="35" t="n"/>
+      <c r="F60" s="35" t="n"/>
+      <c r="G60" s="35" t="n"/>
+      <c r="I60" s="26" t="inlineStr">
         <is>
           <t>Beauty renders at 4K with Movie Render Queue</t>
         </is>
       </c>
-      <c r="J60" s="25" t="inlineStr">
+      <c r="J60" s="26" t="inlineStr">
         <is>
           <t>Breakdown renders</t>
         </is>
       </c>
-      <c r="K60" s="26" t="inlineStr">
+      <c r="K60" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="L60" s="26" t="inlineStr">
+      <c r="L60" s="27" t="inlineStr">
         <is>
           <t>Day off</t>
         </is>
       </c>
-      <c r="M60" s="25" t="inlineStr">
+      <c r="M60" s="26" t="inlineStr">
         <is>
           <t>Marmoset turntables for H1, H2, H6 and a prop sheet</t>
         </is>
       </c>
-      <c r="N60" s="25" t="inlineStr">
+      <c r="N60" s="26" t="inlineStr">
         <is>
           <t>Edit the 30 to 45 second flythrough in Blender's Video Sequencer</t>
         </is>
       </c>
-      <c r="O60" s="25" t="inlineStr">
+      <c r="O60" s="26" t="inlineStr">
         <is>
           <t>Lay out and publish the ArtStation post with breakdown text</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="28" t="inlineStr">
+      <c r="A61" s="30" t="inlineStr">
         <is>
           <t>P10 Glass shards scatter, 8 pieces</t>
         </is>
       </c>
-      <c r="C61" s="33" t="n"/>
-      <c r="D61" s="33" t="n"/>
-      <c r="E61" s="33" t="n"/>
-      <c r="F61" s="33" t="n"/>
-      <c r="G61" s="33" t="n"/>
-      <c r="I61" s="34" t="n"/>
-      <c r="J61" s="34" t="n"/>
-      <c r="K61" s="34" t="n"/>
-      <c r="L61" s="34" t="n"/>
-      <c r="M61" s="34" t="n"/>
-      <c r="N61" s="34" t="n"/>
-      <c r="O61" s="34" t="n"/>
+      <c r="B61" s="29" t="inlineStr">
+        <is>
+          <t>5 to 20</t>
+        </is>
+      </c>
+      <c r="C61" s="35" t="n"/>
+      <c r="D61" s="35" t="n"/>
+      <c r="E61" s="35" t="n"/>
+      <c r="F61" s="35" t="n"/>
+      <c r="G61" s="35" t="n"/>
+      <c r="I61" s="36" t="n"/>
+      <c r="J61" s="36" t="n"/>
+      <c r="K61" s="36" t="n"/>
+      <c r="L61" s="36" t="n"/>
+      <c r="M61" s="36" t="n"/>
+      <c r="N61" s="36" t="n"/>
+      <c r="O61" s="36" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="28" t="inlineStr">
+      <c r="A62" s="30" t="inlineStr">
         <is>
           <t>P11 Dead branches, 5 variants</t>
         </is>
       </c>
-      <c r="C62" s="33" t="n"/>
-      <c r="D62" s="33" t="n"/>
-      <c r="E62" s="33" t="n"/>
-      <c r="F62" s="33" t="n"/>
-      <c r="G62" s="33" t="n"/>
+      <c r="B62" s="29" t="inlineStr">
+        <is>
+          <t>50 to 200</t>
+        </is>
+      </c>
+      <c r="C62" s="35" t="n"/>
+      <c r="D62" s="35" t="n"/>
+      <c r="E62" s="35" t="n"/>
+      <c r="F62" s="35" t="n"/>
+      <c r="G62" s="35" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="28" t="inlineStr">
+      <c r="A63" s="30" t="inlineStr">
         <is>
           <t>P12 Corrugated sheet, bent</t>
         </is>
       </c>
-      <c r="C63" s="33" t="n"/>
-      <c r="D63" s="33" t="n"/>
-      <c r="E63" s="33" t="n"/>
-      <c r="F63" s="33" t="n"/>
-      <c r="G63" s="33" t="n"/>
+      <c r="B63" s="29" t="inlineStr">
+        <is>
+          <t>80 x 200</t>
+        </is>
+      </c>
+      <c r="C63" s="35" t="n"/>
+      <c r="D63" s="35" t="n"/>
+      <c r="E63" s="35" t="n"/>
+      <c r="F63" s="35" t="n"/>
+      <c r="G63" s="35" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="28" t="inlineStr">
+      <c r="A64" s="30" t="inlineStr">
         <is>
           <t>P13 Rusted barrel or drum, on its side</t>
         </is>
       </c>
-      <c r="C64" s="33" t="n"/>
-      <c r="D64" s="33" t="n"/>
-      <c r="E64" s="33" t="n"/>
-      <c r="F64" s="33" t="n"/>
-      <c r="G64" s="33" t="n"/>
+      <c r="B64" s="29" t="inlineStr">
+        <is>
+          <t>60 diameter</t>
+        </is>
+      </c>
+      <c r="C64" s="35" t="n"/>
+      <c r="D64" s="35" t="n"/>
+      <c r="E64" s="35" t="n"/>
+      <c r="F64" s="35" t="n"/>
+      <c r="G64" s="35" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="28" t="inlineStr">
+      <c r="A65" s="30" t="inlineStr">
         <is>
           <t>P14 Crate, broken</t>
         </is>
       </c>
-      <c r="C65" s="33" t="n"/>
-      <c r="D65" s="33" t="n"/>
-      <c r="E65" s="33" t="n"/>
-      <c r="F65" s="33" t="n"/>
-      <c r="G65" s="33" t="n"/>
+      <c r="B65" s="29" t="inlineStr">
+        <is>
+          <t>60 x 60</t>
+        </is>
+      </c>
+      <c r="C65" s="35" t="n"/>
+      <c r="D65" s="35" t="n"/>
+      <c r="E65" s="35" t="n"/>
+      <c r="F65" s="35" t="n"/>
+      <c r="G65" s="35" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="28" t="inlineStr">
+      <c r="A66" s="30" t="inlineStr">
         <is>
           <t>P15 Plastic litter: bags, bottles, cans</t>
         </is>
       </c>
-      <c r="C66" s="33" t="n"/>
-      <c r="D66" s="33" t="n"/>
-      <c r="E66" s="33" t="n"/>
-      <c r="F66" s="33" t="n"/>
-      <c r="G66" s="33" t="n"/>
+      <c r="B66" s="29" t="inlineStr">
+        <is>
+          <t>5 to 40</t>
+        </is>
+      </c>
+      <c r="C66" s="35" t="n"/>
+      <c r="D66" s="35" t="n"/>
+      <c r="E66" s="35" t="n"/>
+      <c r="F66" s="35" t="n"/>
+      <c r="G66" s="35" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="28" t="inlineStr">
+      <c r="A67" s="30" t="inlineStr">
         <is>
           <t>P16 Paper and cardboard scraps</t>
         </is>
       </c>
-      <c r="C67" s="33" t="n"/>
-      <c r="D67" s="33" t="n"/>
-      <c r="E67" s="33" t="n"/>
-      <c r="F67" s="33" t="n"/>
-      <c r="G67" s="33" t="n"/>
+      <c r="B67" s="29" t="inlineStr">
+        <is>
+          <t>10 to 50</t>
+        </is>
+      </c>
+      <c r="C67" s="35" t="n"/>
+      <c r="D67" s="35" t="n"/>
+      <c r="E67" s="35" t="n"/>
+      <c r="F67" s="35" t="n"/>
+      <c r="G67" s="35" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="28" t="inlineStr">
+      <c r="A68" s="30" t="inlineStr">
         <is>
           <t>P17 Wall-mounted junction box</t>
         </is>
       </c>
-      <c r="C68" s="33" t="n"/>
-      <c r="D68" s="33" t="n"/>
-      <c r="E68" s="33" t="n"/>
-      <c r="F68" s="33" t="n"/>
-      <c r="G68" s="33" t="n"/>
+      <c r="B68" s="29" t="inlineStr">
+        <is>
+          <t>30 x 40</t>
+        </is>
+      </c>
+      <c r="C68" s="35" t="n"/>
+      <c r="D68" s="35" t="n"/>
+      <c r="E68" s="35" t="n"/>
+      <c r="F68" s="35" t="n"/>
+      <c r="G68" s="35" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="28" t="inlineStr">
+      <c r="A69" s="30" t="inlineStr">
         <is>
           <t>P18 Old wall lamp bracket</t>
         </is>
       </c>
-      <c r="C69" s="33" t="n"/>
-      <c r="D69" s="33" t="n"/>
-      <c r="E69" s="33" t="n"/>
-      <c r="F69" s="33" t="n"/>
-      <c r="G69" s="33" t="n"/>
+      <c r="B69" s="29" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="C69" s="35" t="n"/>
+      <c r="D69" s="35" t="n"/>
+      <c r="E69" s="35" t="n"/>
+      <c r="F69" s="35" t="n"/>
+      <c r="G69" s="35" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="28" t="inlineStr">
+      <c r="A70" s="30" t="inlineStr">
         <is>
           <t>P19 Fallen roof slates</t>
         </is>
       </c>
-      <c r="C70" s="33" t="n"/>
-      <c r="D70" s="33" t="n"/>
-      <c r="E70" s="33" t="n"/>
-      <c r="F70" s="33" t="n"/>
-      <c r="G70" s="33" t="n"/>
+      <c r="B70" s="29" t="inlineStr">
+        <is>
+          <t>25 x 50</t>
+        </is>
+      </c>
+      <c r="C70" s="35" t="n"/>
+      <c r="D70" s="35" t="n"/>
+      <c r="E70" s="35" t="n"/>
+      <c r="F70" s="35" t="n"/>
+      <c r="G70" s="35" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="28" t="inlineStr">
+      <c r="A71" s="30" t="inlineStr">
         <is>
           <t>P20 Pallet, rotten</t>
         </is>
       </c>
-      <c r="C71" s="33" t="n"/>
-      <c r="D71" s="33" t="n"/>
-      <c r="E71" s="33" t="n"/>
-      <c r="F71" s="33" t="n"/>
-      <c r="G71" s="33" t="n"/>
+      <c r="B71" s="29" t="inlineStr">
+        <is>
+          <t>120 x 100</t>
+        </is>
+      </c>
+      <c r="C71" s="35" t="n"/>
+      <c r="D71" s="35" t="n"/>
+      <c r="E71" s="35" t="n"/>
+      <c r="F71" s="35" t="n"/>
+      <c r="G71" s="35" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="28" t="inlineStr">
+      <c r="A72" s="30" t="inlineStr">
         <is>
           <t>P21 Wire mesh panel, crumpled</t>
         </is>
       </c>
-      <c r="C72" s="33" t="n"/>
-      <c r="D72" s="33" t="n"/>
-      <c r="E72" s="33" t="n"/>
-      <c r="F72" s="33" t="n"/>
-      <c r="G72" s="33" t="n"/>
+      <c r="B72" s="29" t="inlineStr">
+        <is>
+          <t>100 x 200</t>
+        </is>
+      </c>
+      <c r="C72" s="35" t="n"/>
+      <c r="D72" s="35" t="n"/>
+      <c r="E72" s="35" t="n"/>
+      <c r="F72" s="35" t="n"/>
+      <c r="G72" s="35" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="28" t="inlineStr">
+      <c r="A73" s="30" t="inlineStr">
         <is>
           <t>P22 Hose or flex pipe, spline</t>
         </is>
       </c>
-      <c r="C73" s="33" t="n"/>
-      <c r="D73" s="33" t="n"/>
-      <c r="E73" s="33" t="n"/>
-      <c r="F73" s="33" t="n"/>
-      <c r="G73" s="33" t="n"/>
+      <c r="B73" s="29" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="C73" s="35" t="n"/>
+      <c r="D73" s="35" t="n"/>
+      <c r="E73" s="35" t="n"/>
+      <c r="F73" s="35" t="n"/>
+      <c r="G73" s="35" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="29" t="inlineStr">
+      <c r="A74" s="31" t="inlineStr">
         <is>
           <t>Vegetation</t>
         </is>
       </c>
-      <c r="B74" s="29" t="n"/>
-      <c r="C74" s="29" t="inlineStr">
+      <c r="B74" s="31" t="inlineStr">
+        <is>
+          <t>Size (cm)</t>
+        </is>
+      </c>
+      <c r="C74" s="31" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="D74" s="29" t="inlineStr">
+      <c r="D74" s="31" t="inlineStr">
         <is>
           <t>Atlas</t>
         </is>
       </c>
-      <c r="E74" s="29" t="inlineStr">
+      <c r="E74" s="31" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="F74" s="29" t="inlineStr">
+      <c r="F74" s="31" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
       </c>
-      <c r="G74" s="29" t="inlineStr">
+      <c r="G74" s="31" t="inlineStr">
         <is>
           <t>Placed</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="30" t="n"/>
-      <c r="B75" s="30" t="n"/>
-      <c r="C75" s="30" t="n"/>
-      <c r="D75" s="30" t="n"/>
-      <c r="E75" s="30" t="n"/>
-      <c r="F75" s="30" t="n"/>
-      <c r="G75" s="30" t="n"/>
+      <c r="A75" s="32" t="n"/>
+      <c r="B75" s="32" t="n"/>
+      <c r="C75" s="32" t="n"/>
+      <c r="D75" s="32" t="n"/>
+      <c r="E75" s="32" t="n"/>
+      <c r="F75" s="32" t="n"/>
+      <c r="G75" s="32" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="28" t="inlineStr">
+      <c r="A76" s="30" t="inlineStr">
         <is>
           <t>F01 Ivy cards and vine splines</t>
         </is>
       </c>
-      <c r="C76" s="33" t="n"/>
-      <c r="D76" s="33" t="n"/>
-      <c r="E76" s="33" t="n"/>
-      <c r="F76" s="33" t="n"/>
-      <c r="G76" s="33" t="n"/>
+      <c r="B76" s="29" t="n"/>
+      <c r="C76" s="35" t="n"/>
+      <c r="D76" s="35" t="n"/>
+      <c r="E76" s="35" t="n"/>
+      <c r="F76" s="35" t="n"/>
+      <c r="G76" s="35" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="28" t="inlineStr">
+      <c r="A77" s="30" t="inlineStr">
         <is>
           <t>F02 Moss clumps, 3 sizes</t>
         </is>
       </c>
-      <c r="C77" s="33" t="n"/>
-      <c r="D77" s="33" t="n"/>
-      <c r="E77" s="33" t="n"/>
-      <c r="F77" s="33" t="n"/>
-      <c r="G77" s="33" t="n"/>
+      <c r="B77" s="29" t="n"/>
+      <c r="C77" s="35" t="n"/>
+      <c r="D77" s="35" t="n"/>
+      <c r="E77" s="35" t="n"/>
+      <c r="F77" s="35" t="n"/>
+      <c r="G77" s="35" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="28" t="inlineStr">
+      <c r="A78" s="30" t="inlineStr">
         <is>
           <t>F03 Grass and weed tufts, 6 variants</t>
         </is>
       </c>
-      <c r="C78" s="33" t="n"/>
-      <c r="D78" s="33" t="n"/>
-      <c r="E78" s="33" t="n"/>
-      <c r="F78" s="33" t="n"/>
-      <c r="G78" s="33" t="n"/>
+      <c r="B78" s="29" t="n"/>
+      <c r="C78" s="35" t="n"/>
+      <c r="D78" s="35" t="n"/>
+      <c r="E78" s="35" t="n"/>
+      <c r="F78" s="35" t="n"/>
+      <c r="G78" s="35" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="28" t="inlineStr">
+      <c r="A79" s="30" t="inlineStr">
         <is>
           <t>F04 Buddleia bush (grows from walls)</t>
         </is>
       </c>
-      <c r="C79" s="33" t="n"/>
-      <c r="D79" s="33" t="n"/>
-      <c r="E79" s="33" t="n"/>
-      <c r="F79" s="33" t="n"/>
-      <c r="G79" s="33" t="n"/>
+      <c r="B79" s="29" t="n"/>
+      <c r="C79" s="35" t="n"/>
+      <c r="D79" s="35" t="n"/>
+      <c r="E79" s="35" t="n"/>
+      <c r="F79" s="35" t="n"/>
+      <c r="G79" s="35" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="28" t="inlineStr">
+      <c r="A80" s="30" t="inlineStr">
         <is>
           <t>F05 Dead leaves scatter</t>
         </is>
       </c>
-      <c r="C80" s="33" t="n"/>
-      <c r="D80" s="33" t="n"/>
-      <c r="E80" s="33" t="n"/>
-      <c r="F80" s="33" t="n"/>
-      <c r="G80" s="33" t="n"/>
+      <c r="B80" s="29" t="n"/>
+      <c r="C80" s="35" t="n"/>
+      <c r="D80" s="35" t="n"/>
+      <c r="E80" s="35" t="n"/>
+      <c r="F80" s="35" t="n"/>
+      <c r="G80" s="35" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="28" t="inlineStr">
+      <c r="A81" s="30" t="inlineStr">
         <is>
           <t>F06 Brambles</t>
         </is>
       </c>
-      <c r="C81" s="33" t="n"/>
-      <c r="D81" s="33" t="n"/>
-      <c r="E81" s="33" t="n"/>
-      <c r="F81" s="33" t="n"/>
-      <c r="G81" s="33" t="n"/>
+      <c r="B81" s="29" t="n"/>
+      <c r="C81" s="35" t="n"/>
+      <c r="D81" s="35" t="n"/>
+      <c r="E81" s="35" t="n"/>
+      <c r="F81" s="35" t="n"/>
+      <c r="G81" s="35" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="28" t="inlineStr">
+      <c r="A82" s="30" t="inlineStr">
         <is>
           <t>F07 Small birch and sycamore saplings</t>
         </is>
       </c>
-      <c r="C82" s="33" t="n"/>
-      <c r="D82" s="33" t="n"/>
-      <c r="E82" s="33" t="n"/>
-      <c r="F82" s="33" t="n"/>
-      <c r="G82" s="33" t="n"/>
+      <c r="B82" s="29" t="n"/>
+      <c r="C82" s="35" t="n"/>
+      <c r="D82" s="35" t="n"/>
+      <c r="E82" s="35" t="n"/>
+      <c r="F82" s="35" t="n"/>
+      <c r="G82" s="35" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="28" t="inlineStr">
+      <c r="A83" s="30" t="inlineStr">
         <is>
           <t>F08 Background trees (far opening)</t>
         </is>
       </c>
-      <c r="C83" s="33" t="n"/>
-      <c r="D83" s="33" t="n"/>
-      <c r="E83" s="33" t="n"/>
-      <c r="F83" s="33" t="n"/>
-      <c r="G83" s="33" t="n"/>
+      <c r="B83" s="29" t="n"/>
+      <c r="C83" s="35" t="n"/>
+      <c r="D83" s="35" t="n"/>
+      <c r="E83" s="35" t="n"/>
+      <c r="F83" s="35" t="n"/>
+      <c r="G83" s="35" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="28" t="inlineStr">
+      <c r="A84" s="30" t="inlineStr">
         <is>
           <t>F09 Roof-edge weeds for the chimney building</t>
         </is>
       </c>
-      <c r="C84" s="33" t="n"/>
-      <c r="D84" s="33" t="n"/>
-      <c r="E84" s="33" t="n"/>
-      <c r="F84" s="33" t="n"/>
-      <c r="G84" s="33" t="n"/>
+      <c r="B84" s="29" t="n"/>
+      <c r="C84" s="35" t="n"/>
+      <c r="D84" s="35" t="n"/>
+      <c r="E84" s="35" t="n"/>
+      <c r="F84" s="35" t="n"/>
+      <c r="G84" s="35" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="28" t="inlineStr">
+      <c r="A85" s="30" t="inlineStr">
         <is>
           <t>F10 Ferns in damp corners</t>
         </is>
       </c>
-      <c r="C85" s="33" t="n"/>
-      <c r="D85" s="33" t="n"/>
-      <c r="E85" s="33" t="n"/>
-      <c r="F85" s="33" t="n"/>
-      <c r="G85" s="33" t="n"/>
+      <c r="B85" s="29" t="n"/>
+      <c r="C85" s="35" t="n"/>
+      <c r="D85" s="35" t="n"/>
+      <c r="E85" s="35" t="n"/>
+      <c r="F85" s="35" t="n"/>
+      <c r="G85" s="35" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="29" t="inlineStr">
+      <c r="A86" s="31" t="inlineStr">
         <is>
           <t>Tile-Textures</t>
         </is>
       </c>
-      <c r="B86" s="29" t="n"/>
-      <c r="C86" s="29" t="inlineStr">
+      <c r="B86" s="31" t="inlineStr">
+        <is>
+          <t>Size (cm)</t>
+        </is>
+      </c>
+      <c r="C86" s="31" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D86" s="29" t="inlineStr">
+      <c r="D86" s="31" t="inlineStr">
         <is>
           <t>Customize</t>
         </is>
       </c>
-      <c r="E86" s="29" t="inlineStr">
+      <c r="E86" s="31" t="inlineStr">
         <is>
           <t>Masks</t>
         </is>
       </c>
-      <c r="F86" s="29" t="inlineStr">
+      <c r="F86" s="31" t="inlineStr">
         <is>
           <t>Bake</t>
         </is>
       </c>
-      <c r="G86" s="29" t="inlineStr">
+      <c r="G86" s="31" t="inlineStr">
         <is>
           <t>In UE5</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="30" t="n"/>
-      <c r="B87" s="30" t="n"/>
-      <c r="C87" s="30" t="n"/>
-      <c r="D87" s="30" t="n"/>
-      <c r="E87" s="30" t="n"/>
-      <c r="F87" s="30" t="n"/>
-      <c r="G87" s="30" t="n"/>
+      <c r="A87" s="32" t="n"/>
+      <c r="B87" s="32" t="n"/>
+      <c r="C87" s="32" t="n"/>
+      <c r="D87" s="32" t="n"/>
+      <c r="E87" s="32" t="n"/>
+      <c r="F87" s="32" t="n"/>
+      <c r="G87" s="32" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="28" t="inlineStr">
+      <c r="A88" s="30" t="inlineStr">
         <is>
           <t>M01 Brick, sooty dark (Victorian, recessed mortar)</t>
         </is>
       </c>
-      <c r="C88" s="33" t="n"/>
-      <c r="D88" s="33" t="n"/>
-      <c r="E88" s="33" t="n"/>
-      <c r="F88" s="33" t="n"/>
-      <c r="G88" s="33" t="n"/>
+      <c r="B88" s="29" t="inlineStr">
+        <is>
+          <t>200 x 200 tile</t>
+        </is>
+      </c>
+      <c r="C88" s="35" t="n"/>
+      <c r="D88" s="35" t="n"/>
+      <c r="E88" s="35" t="n"/>
+      <c r="F88" s="35" t="n"/>
+      <c r="G88" s="35" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="28" t="inlineStr">
+      <c r="A89" s="30" t="inlineStr">
         <is>
           <t>M02 Brick, grey limewash peeling to red brick</t>
         </is>
       </c>
-      <c r="C89" s="33" t="n"/>
-      <c r="D89" s="33" t="n"/>
-      <c r="E89" s="33" t="n"/>
-      <c r="F89" s="33" t="n"/>
-      <c r="G89" s="33" t="n"/>
+      <c r="B89" s="29" t="inlineStr">
+        <is>
+          <t>200 x 200 tile</t>
+        </is>
+      </c>
+      <c r="C89" s="35" t="n"/>
+      <c r="D89" s="35" t="n"/>
+      <c r="E89" s="35" t="n"/>
+      <c r="F89" s="35" t="n"/>
+      <c r="G89" s="35" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="28" t="inlineStr">
+      <c r="A90" s="30" t="inlineStr">
         <is>
           <t>M03 Brick, red clean (background)</t>
         </is>
       </c>
-      <c r="C90" s="33" t="n"/>
-      <c r="D90" s="33" t="n"/>
-      <c r="E90" s="33" t="n"/>
-      <c r="F90" s="33" t="n"/>
-      <c r="G90" s="33" t="n"/>
+      <c r="B90" s="29" t="inlineStr">
+        <is>
+          <t>200 x 200 tile</t>
+        </is>
+      </c>
+      <c r="C90" s="35" t="n"/>
+      <c r="D90" s="35" t="n"/>
+      <c r="E90" s="35" t="n"/>
+      <c r="F90" s="35" t="n"/>
+      <c r="G90" s="35" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="28" t="inlineStr">
+      <c r="A91" s="30" t="inlineStr">
         <is>
           <t>M04 Brick infill, mismatched</t>
         </is>
       </c>
-      <c r="C91" s="33" t="n"/>
-      <c r="D91" s="33" t="n"/>
-      <c r="E91" s="33" t="n"/>
-      <c r="F91" s="33" t="n"/>
-      <c r="G91" s="33" t="n"/>
+      <c r="B91" s="29" t="inlineStr">
+        <is>
+          <t>200 x 200 tile</t>
+        </is>
+      </c>
+      <c r="C91" s="35" t="n"/>
+      <c r="D91" s="35" t="n"/>
+      <c r="E91" s="35" t="n"/>
+      <c r="F91" s="35" t="n"/>
+      <c r="G91" s="35" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="28" t="inlineStr">
+      <c r="A92" s="30" t="inlineStr">
         <is>
           <t>M05 Ground setts under mud</t>
         </is>
       </c>
-      <c r="C92" s="33" t="n"/>
-      <c r="D92" s="33" t="n"/>
-      <c r="E92" s="33" t="n"/>
-      <c r="F92" s="33" t="n"/>
-      <c r="G92" s="33" t="n"/>
+      <c r="B92" s="29" t="inlineStr">
+        <is>
+          <t>200 x 200 tile</t>
+        </is>
+      </c>
+      <c r="C92" s="35" t="n"/>
+      <c r="D92" s="35" t="n"/>
+      <c r="E92" s="35" t="n"/>
+      <c r="F92" s="35" t="n"/>
+      <c r="G92" s="35" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="28" t="inlineStr">
+      <c r="A93" s="30" t="inlineStr">
         <is>
           <t>M06 Mud and dirt with organic debris</t>
         </is>
       </c>
-      <c r="C93" s="33" t="n"/>
-      <c r="D93" s="33" t="n"/>
-      <c r="E93" s="33" t="n"/>
-      <c r="F93" s="33" t="n"/>
-      <c r="G93" s="33" t="n"/>
+      <c r="B93" s="29" t="inlineStr">
+        <is>
+          <t>200 x 200 tile</t>
+        </is>
+      </c>
+      <c r="C93" s="35" t="n"/>
+      <c r="D93" s="35" t="n"/>
+      <c r="E93" s="35" t="n"/>
+      <c r="F93" s="35" t="n"/>
+      <c r="G93" s="35" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="28" t="inlineStr">
+      <c r="A94" s="30" t="inlineStr">
         <is>
           <t>M07 Concrete, weathered</t>
         </is>
       </c>
-      <c r="C94" s="33" t="n"/>
-      <c r="D94" s="33" t="n"/>
-      <c r="E94" s="33" t="n"/>
-      <c r="F94" s="33" t="n"/>
-      <c r="G94" s="33" t="n"/>
+      <c r="B94" s="29" t="inlineStr">
+        <is>
+          <t>200 x 200 tile</t>
+        </is>
+      </c>
+      <c r="C94" s="35" t="n"/>
+      <c r="D94" s="35" t="n"/>
+      <c r="E94" s="35" t="n"/>
+      <c r="F94" s="35" t="n"/>
+      <c r="G94" s="35" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="28" t="inlineStr">
+      <c r="A95" s="30" t="inlineStr">
         <is>
           <t>M08 Moss and algae</t>
         </is>
       </c>
-      <c r="C95" s="33" t="n"/>
-      <c r="D95" s="33" t="n"/>
-      <c r="E95" s="33" t="n"/>
-      <c r="F95" s="33" t="n"/>
-      <c r="G95" s="33" t="n"/>
+      <c r="B95" s="29" t="inlineStr">
+        <is>
+          <t>100 x 100 tile</t>
+        </is>
+      </c>
+      <c r="C95" s="35" t="n"/>
+      <c r="D95" s="35" t="n"/>
+      <c r="E95" s="35" t="n"/>
+      <c r="F95" s="35" t="n"/>
+      <c r="G95" s="35" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="28" t="inlineStr">
+      <c r="A96" s="30" t="inlineStr">
         <is>
           <t>M09 Timber, painted and peeling (red, green)</t>
         </is>
       </c>
-      <c r="C96" s="33" t="n"/>
-      <c r="D96" s="33" t="n"/>
-      <c r="E96" s="33" t="n"/>
-      <c r="F96" s="33" t="n"/>
-      <c r="G96" s="33" t="n"/>
+      <c r="B96" s="29" t="inlineStr">
+        <is>
+          <t>200 x 200 tile</t>
+        </is>
+      </c>
+      <c r="C96" s="35" t="n"/>
+      <c r="D96" s="35" t="n"/>
+      <c r="E96" s="35" t="n"/>
+      <c r="F96" s="35" t="n"/>
+      <c r="G96" s="35" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="28" t="inlineStr">
+      <c r="A97" s="30" t="inlineStr">
         <is>
           <t>M10 Rusted painted metal</t>
         </is>
       </c>
-      <c r="C97" s="33" t="n"/>
-      <c r="D97" s="33" t="n"/>
-      <c r="E97" s="33" t="n"/>
-      <c r="F97" s="33" t="n"/>
-      <c r="G97" s="33" t="n"/>
+      <c r="B97" s="29" t="inlineStr">
+        <is>
+          <t>100 x 100 tile</t>
+        </is>
+      </c>
+      <c r="C97" s="35" t="n"/>
+      <c r="D97" s="35" t="n"/>
+      <c r="E97" s="35" t="n"/>
+      <c r="F97" s="35" t="n"/>
+      <c r="G97" s="35" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="29" t="inlineStr">
+      <c r="A98" s="31" t="inlineStr">
         <is>
           <t>Trim sheets</t>
         </is>
       </c>
-      <c r="B98" s="29" t="n"/>
-      <c r="C98" s="29" t="inlineStr">
+      <c r="B98" s="31" t="inlineStr">
+        <is>
+          <t>Size (cm)</t>
+        </is>
+      </c>
+      <c r="C98" s="31" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="D98" s="29" t="inlineStr">
+      <c r="D98" s="31" t="inlineStr">
         <is>
           <t>Bake</t>
         </is>
       </c>
-      <c r="E98" s="29" t="inlineStr">
+      <c r="E98" s="31" t="inlineStr">
         <is>
           <t>Texture</t>
         </is>
       </c>
-      <c r="F98" s="29" t="inlineStr">
+      <c r="F98" s="31" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="G98" s="29" t="inlineStr">
+      <c r="G98" s="31" t="inlineStr">
         <is>
           <t>In UE5</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="30" t="n"/>
-      <c r="B99" s="30" t="n"/>
-      <c r="C99" s="30" t="n"/>
-      <c r="D99" s="30" t="n"/>
-      <c r="E99" s="30" t="n"/>
-      <c r="F99" s="30" t="n"/>
-      <c r="G99" s="30" t="n"/>
+      <c r="A99" s="32" t="n"/>
+      <c r="B99" s="32" t="n"/>
+      <c r="C99" s="32" t="n"/>
+      <c r="D99" s="32" t="n"/>
+      <c r="E99" s="32" t="n"/>
+      <c r="F99" s="32" t="n"/>
+      <c r="G99" s="32" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="28" t="inlineStr">
+      <c r="A100" s="30" t="inlineStr">
         <is>
           <t>T01 Stone trim sheet</t>
         </is>
       </c>
-      <c r="C100" s="33" t="n"/>
-      <c r="D100" s="33" t="n"/>
-      <c r="E100" s="33" t="n"/>
-      <c r="F100" s="33" t="n"/>
-      <c r="G100" s="33" t="n"/>
+      <c r="B100" s="29" t="inlineStr">
+        <is>
+          <t>2048 px, 10.24 px/cm</t>
+        </is>
+      </c>
+      <c r="C100" s="35" t="n"/>
+      <c r="D100" s="35" t="n"/>
+      <c r="E100" s="35" t="n"/>
+      <c r="F100" s="35" t="n"/>
+      <c r="G100" s="35" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="28" t="inlineStr">
+      <c r="A101" s="30" t="inlineStr">
         <is>
           <t>T02 Metal trim sheet</t>
         </is>
       </c>
-      <c r="C101" s="33" t="n"/>
-      <c r="D101" s="33" t="n"/>
-      <c r="E101" s="33" t="n"/>
-      <c r="F101" s="33" t="n"/>
-      <c r="G101" s="33" t="n"/>
+      <c r="B101" s="29" t="inlineStr">
+        <is>
+          <t>2048 px, 10.24 px/cm</t>
+        </is>
+      </c>
+      <c r="C101" s="35" t="n"/>
+      <c r="D101" s="35" t="n"/>
+      <c r="E101" s="35" t="n"/>
+      <c r="F101" s="35" t="n"/>
+      <c r="G101" s="35" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="28" t="inlineStr">
+      <c r="A102" s="30" t="inlineStr">
         <is>
           <t>T03 Timber trim sheet</t>
         </is>
       </c>
-      <c r="C102" s="33" t="n"/>
-      <c r="D102" s="33" t="n"/>
-      <c r="E102" s="33" t="n"/>
-      <c r="F102" s="33" t="n"/>
-      <c r="G102" s="33" t="n"/>
+      <c r="B102" s="29" t="inlineStr">
+        <is>
+          <t>2048 px, 10.24 px/cm</t>
+        </is>
+      </c>
+      <c r="C102" s="35" t="n"/>
+      <c r="D102" s="35" t="n"/>
+      <c r="E102" s="35" t="n"/>
+      <c r="F102" s="35" t="n"/>
+      <c r="G102" s="35" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="29" t="inlineStr">
+      <c r="A103" s="31" t="inlineStr">
         <is>
           <t>Decals</t>
         </is>
       </c>
-      <c r="B103" s="29" t="n"/>
-      <c r="C103" s="29" t="inlineStr">
+      <c r="B103" s="31" t="inlineStr">
+        <is>
+          <t>Size (cm)</t>
+        </is>
+      </c>
+      <c r="C103" s="31" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D103" s="29" t="inlineStr">
+      <c r="D103" s="31" t="inlineStr">
         <is>
           <t>Bake</t>
         </is>
       </c>
-      <c r="E103" s="29" t="inlineStr">
+      <c r="E103" s="31" t="inlineStr">
         <is>
           <t>Texture</t>
         </is>
       </c>
-      <c r="F103" s="29" t="inlineStr">
+      <c r="F103" s="31" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="G103" s="29" t="inlineStr">
+      <c r="G103" s="31" t="inlineStr">
         <is>
           <t>Placed</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="30" t="n"/>
-      <c r="B104" s="30" t="n"/>
-      <c r="C104" s="30" t="n"/>
-      <c r="D104" s="30" t="n"/>
-      <c r="E104" s="30" t="n"/>
-      <c r="F104" s="30" t="n"/>
-      <c r="G104" s="30" t="n"/>
+      <c r="A104" s="32" t="n"/>
+      <c r="B104" s="32" t="n"/>
+      <c r="C104" s="32" t="n"/>
+      <c r="D104" s="32" t="n"/>
+      <c r="E104" s="32" t="n"/>
+      <c r="F104" s="32" t="n"/>
+      <c r="G104" s="32" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="28" t="inlineStr">
+      <c r="A105" s="30" t="inlineStr">
         <is>
           <t>X01 Water leaks and streaks under sills and pipes</t>
         </is>
       </c>
-      <c r="C105" s="33" t="n"/>
-      <c r="D105" s="33" t="n"/>
-      <c r="E105" s="33" t="n"/>
-      <c r="F105" s="33" t="n"/>
-      <c r="G105" s="33" t="n"/>
+      <c r="B105" s="29" t="n"/>
+      <c r="C105" s="35" t="n"/>
+      <c r="D105" s="35" t="n"/>
+      <c r="E105" s="35" t="n"/>
+      <c r="F105" s="35" t="n"/>
+      <c r="G105" s="35" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="28" t="inlineStr">
+      <c r="A106" s="30" t="inlineStr">
         <is>
           <t>X02 Soot and grime gradients up from the ground</t>
         </is>
       </c>
-      <c r="C106" s="33" t="n"/>
-      <c r="D106" s="33" t="n"/>
-      <c r="E106" s="33" t="n"/>
-      <c r="F106" s="33" t="n"/>
-      <c r="G106" s="33" t="n"/>
+      <c r="B106" s="29" t="n"/>
+      <c r="C106" s="35" t="n"/>
+      <c r="D106" s="35" t="n"/>
+      <c r="E106" s="35" t="n"/>
+      <c r="F106" s="35" t="n"/>
+      <c r="G106" s="35" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="28" t="inlineStr">
+      <c r="A107" s="30" t="inlineStr">
         <is>
           <t>X03 Moss and algae patches</t>
         </is>
       </c>
-      <c r="C107" s="33" t="n"/>
-      <c r="D107" s="33" t="n"/>
-      <c r="E107" s="33" t="n"/>
-      <c r="F107" s="33" t="n"/>
-      <c r="G107" s="33" t="n"/>
+      <c r="B107" s="29" t="n"/>
+      <c r="C107" s="35" t="n"/>
+      <c r="D107" s="35" t="n"/>
+      <c r="E107" s="35" t="n"/>
+      <c r="F107" s="35" t="n"/>
+      <c r="G107" s="35" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="28" t="inlineStr">
+      <c r="A108" s="30" t="inlineStr">
         <is>
           <t>X04 Brick damage, spalling and cracks</t>
         </is>
       </c>
-      <c r="C108" s="33" t="n"/>
-      <c r="D108" s="33" t="n"/>
-      <c r="E108" s="33" t="n"/>
-      <c r="F108" s="33" t="n"/>
-      <c r="G108" s="33" t="n"/>
+      <c r="B108" s="29" t="n"/>
+      <c r="C108" s="35" t="n"/>
+      <c r="D108" s="35" t="n"/>
+      <c r="E108" s="35" t="n"/>
+      <c r="F108" s="35" t="n"/>
+      <c r="G108" s="35" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="28" t="inlineStr">
+      <c r="A109" s="30" t="inlineStr">
         <is>
           <t>X05 Peeling paint edges (right wall)</t>
         </is>
       </c>
-      <c r="C109" s="33" t="n"/>
-      <c r="D109" s="33" t="n"/>
-      <c r="E109" s="33" t="n"/>
-      <c r="F109" s="33" t="n"/>
-      <c r="G109" s="33" t="n"/>
+      <c r="B109" s="29" t="n"/>
+      <c r="C109" s="35" t="n"/>
+      <c r="D109" s="35" t="n"/>
+      <c r="E109" s="35" t="n"/>
+      <c r="F109" s="35" t="n"/>
+      <c r="G109" s="35" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="28" t="inlineStr">
+      <c r="A110" s="30" t="inlineStr">
         <is>
           <t>X06 Rust bleed from metal fixings</t>
         </is>
       </c>
-      <c r="C110" s="33" t="n"/>
-      <c r="D110" s="33" t="n"/>
-      <c r="E110" s="33" t="n"/>
-      <c r="F110" s="33" t="n"/>
-      <c r="G110" s="33" t="n"/>
+      <c r="B110" s="29" t="n"/>
+      <c r="C110" s="35" t="n"/>
+      <c r="D110" s="35" t="n"/>
+      <c r="E110" s="35" t="n"/>
+      <c r="F110" s="35" t="n"/>
+      <c r="G110" s="35" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="28" t="inlineStr">
+      <c r="A111" s="30" t="inlineStr">
         <is>
           <t>X07 Puddle and wet-ground patches</t>
         </is>
       </c>
-      <c r="C111" s="33" t="n"/>
-      <c r="D111" s="33" t="n"/>
-      <c r="E111" s="33" t="n"/>
-      <c r="F111" s="33" t="n"/>
-      <c r="G111" s="33" t="n"/>
+      <c r="B111" s="29" t="n"/>
+      <c r="C111" s="35" t="n"/>
+      <c r="D111" s="35" t="n"/>
+      <c r="E111" s="35" t="n"/>
+      <c r="F111" s="35" t="n"/>
+      <c r="G111" s="35" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="28" t="inlineStr">
+      <c r="A112" s="30" t="inlineStr">
         <is>
           <t>X08 Oil stains and mud tracks</t>
         </is>
       </c>
-      <c r="C112" s="33" t="n"/>
-      <c r="D112" s="33" t="n"/>
-      <c r="E112" s="33" t="n"/>
-      <c r="F112" s="33" t="n"/>
-      <c r="G112" s="33" t="n"/>
+      <c r="B112" s="29" t="n"/>
+      <c r="C112" s="35" t="n"/>
+      <c r="D112" s="35" t="n"/>
+      <c r="E112" s="35" t="n"/>
+      <c r="F112" s="35" t="n"/>
+      <c r="G112" s="35" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="28" t="inlineStr">
+      <c r="A113" s="30" t="inlineStr">
         <is>
           <t>X09 Old painted signage, faded</t>
         </is>
       </c>
-      <c r="C113" s="33" t="n"/>
-      <c r="D113" s="33" t="n"/>
-      <c r="E113" s="33" t="n"/>
-      <c r="F113" s="33" t="n"/>
-      <c r="G113" s="33" t="n"/>
+      <c r="B113" s="29" t="n"/>
+      <c r="C113" s="35" t="n"/>
+      <c r="D113" s="35" t="n"/>
+      <c r="E113" s="35" t="n"/>
+      <c r="F113" s="35" t="n"/>
+      <c r="G113" s="35" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="35" t="n"/>
-      <c r="B116" s="28" t="inlineStr">
+      <c r="A116" s="37" t="n"/>
+      <c r="B116" s="30" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="36" t="n"/>
-      <c r="B117" s="28" t="inlineStr">
+      <c r="A117" s="38" t="n"/>
+      <c r="B117" s="30" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="33" t="n"/>
-      <c r="B118" s="28" t="inlineStr">
+      <c r="A118" s="35" t="n"/>
+      <c r="B118" s="30" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="37" t="inlineStr">
+      <c r="A120" s="39" t="inlineStr">
         <is>
           <t>Change a stage cell's fill colour to update its status.</t>
         </is>
@@ -3732,4 +4159,552 @@
   <pageSetup orientation="landscape" fitToHeight="0" pageOrder="overThenDown" cellComments="atEnd"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" style="17" min="1" max="1"/>
+    <col width="14" customWidth="1" style="17" min="2" max="2"/>
+    <col width="14" customWidth="1" style="17" min="3" max="3"/>
+    <col width="18" customWidth="1" style="17" min="4" max="4"/>
+    <col width="52" customWidth="1" style="17" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
+        <is>
+          <t>Reference breakdown · 1:1 scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>Estimates from human-scale anchors (100 cm handrail, 18 cm risers, 210-260 cm doors, Victorian brick coursing). Confirm by camera-matching the photo in Blender.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="31" t="inlineStr">
+        <is>
+          <t>Element</t>
+        </is>
+      </c>
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>Width (cm)</t>
+        </is>
+      </c>
+      <c r="C4" s="31" t="inlineStr">
+        <is>
+          <t>Height (cm)</t>
+        </is>
+      </c>
+      <c r="D4" s="31" t="inlineStr">
+        <is>
+          <t>Depth (cm)</t>
+        </is>
+      </c>
+      <c r="E4" s="31" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="40" t="inlineStr">
+        <is>
+          <t>Alley, wall to wall</t>
+        </is>
+      </c>
+      <c r="B5" s="40" t="n">
+        <v>500</v>
+      </c>
+      <c r="C5" s="40" t="n"/>
+      <c r="D5" s="40" t="inlineStr">
+        <is>
+          <t>4000 visible length</t>
+        </is>
+      </c>
+      <c r="E5" s="40" t="inlineStr">
+        <is>
+          <t>about 400 clear walkway beside the light well</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>Left mill height</t>
+        </is>
+      </c>
+      <c r="B6" s="41" t="n"/>
+      <c r="C6" s="41" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D6" s="41" t="n"/>
+      <c r="E6" s="41" t="inlineStr">
+        <is>
+          <t>5 storeys at 400 floor to floor, plus parapet</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="40" t="inlineStr">
+        <is>
+          <t>Right building height</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="n"/>
+      <c r="C7" s="40" t="n">
+        <v>1900</v>
+      </c>
+      <c r="D7" s="40" t="n"/>
+      <c r="E7" s="40" t="inlineStr">
+        <is>
+          <t>5 storeys at about 380 floor to floor</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="41" t="inlineStr">
+        <is>
+          <t>Brick (Victorian imperial)</t>
+        </is>
+      </c>
+      <c r="B8" s="41" t="n">
+        <v>23</v>
+      </c>
+      <c r="C8" s="41" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="D8" s="41" t="n">
+        <v>11</v>
+      </c>
+      <c r="E8" s="41" t="inlineStr">
+        <is>
+          <t>1 cm joints, so 8.6 cm per course, about 12 courses per metre</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="40" t="inlineStr">
+        <is>
+          <t>Left pilaster</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="n">
+        <v>60</v>
+      </c>
+      <c r="C9" s="40" t="inlineStr">
+        <is>
+          <t>full height</t>
+        </is>
+      </c>
+      <c r="D9" s="40" t="inlineStr">
+        <is>
+          <t>25 projection</t>
+        </is>
+      </c>
+      <c r="E9" s="40" t="inlineStr">
+        <is>
+          <t>every 400 along the wall</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="41" t="inlineStr">
+        <is>
+          <t>Left blind arch recess</t>
+        </is>
+      </c>
+      <c r="B10" s="41" t="n">
+        <v>200</v>
+      </c>
+      <c r="C10" s="41" t="n">
+        <v>550</v>
+      </c>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>25 recess</t>
+        </is>
+      </c>
+      <c r="E10" s="41" t="inlineStr">
+        <is>
+          <t>round head, bricked-up infill</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="40" t="inlineStr">
+        <is>
+          <t>Left arched loading door</t>
+        </is>
+      </c>
+      <c r="B11" s="40" t="n">
+        <v>240</v>
+      </c>
+      <c r="C11" s="40" t="n">
+        <v>320</v>
+      </c>
+      <c r="D11" s="40" t="inlineStr">
+        <is>
+          <t>40 reveal</t>
+        </is>
+      </c>
+      <c r="E11" s="40" t="inlineStr">
+        <is>
+          <t>rusted sheet doors</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="41" t="inlineStr">
+        <is>
+          <t>Right window opening</t>
+        </is>
+      </c>
+      <c r="B12" s="41" t="n">
+        <v>140</v>
+      </c>
+      <c r="C12" s="41" t="n">
+        <v>220</v>
+      </c>
+      <c r="D12" s="41" t="inlineStr">
+        <is>
+          <t>30 reveal</t>
+        </is>
+      </c>
+      <c r="E12" s="41" t="inlineStr">
+        <is>
+          <t>steel frame, panes about 25 x 35</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="40" t="inlineStr">
+        <is>
+          <t>Right window bay spacing</t>
+        </is>
+      </c>
+      <c r="B13" s="40" t="n">
+        <v>300</v>
+      </c>
+      <c r="C13" s="40" t="n">
+        <v>380</v>
+      </c>
+      <c r="D13" s="40" t="n"/>
+      <c r="E13" s="40" t="inlineStr">
+        <is>
+          <t>160 of brick pier between openings</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="41" t="inlineStr">
+        <is>
+          <t>Stone sill</t>
+        </is>
+      </c>
+      <c r="B14" s="41" t="n">
+        <v>160</v>
+      </c>
+      <c r="C14" s="41" t="n">
+        <v>15</v>
+      </c>
+      <c r="D14" s="41" t="n">
+        <v>20</v>
+      </c>
+      <c r="E14" s="41" t="inlineStr">
+        <is>
+          <t>5 projection, drip groove</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="40" t="inlineStr">
+        <is>
+          <t>Stone lintel</t>
+        </is>
+      </c>
+      <c r="B15" s="40" t="n">
+        <v>170</v>
+      </c>
+      <c r="C15" s="40" t="n">
+        <v>30</v>
+      </c>
+      <c r="D15" s="40" t="n">
+        <v>30</v>
+      </c>
+      <c r="E15" s="40" t="inlineStr">
+        <is>
+          <t>flush or 2 projection</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="41" t="inlineStr">
+        <is>
+          <t>Right mossy ledge / plinth</t>
+        </is>
+      </c>
+      <c r="B16" s="41" t="inlineStr">
+        <is>
+          <t>runs wall</t>
+        </is>
+      </c>
+      <c r="C16" s="41" t="n">
+        <v>50</v>
+      </c>
+      <c r="D16" s="41" t="n">
+        <v>60</v>
+      </c>
+      <c r="E16" s="41" t="inlineStr">
+        <is>
+          <t>top surface takes world-aligned moss</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="40" t="inlineStr">
+        <is>
+          <t>Basement light well</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="n">
+        <v>120</v>
+      </c>
+      <c r="C17" s="40" t="inlineStr">
+        <is>
+          <t>200 drop</t>
+        </is>
+      </c>
+      <c r="D17" s="40" t="n">
+        <v>380</v>
+      </c>
+      <c r="E17" s="40" t="inlineStr">
+        <is>
+          <t>11 risers at 18, treads 28</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="41" t="inlineStr">
+        <is>
+          <t>Handrail</t>
+        </is>
+      </c>
+      <c r="B18" s="41" t="inlineStr">
+        <is>
+          <t>4.2 diameter</t>
+        </is>
+      </c>
+      <c r="C18" s="41" t="n">
+        <v>100</v>
+      </c>
+      <c r="D18" s="41" t="n"/>
+      <c r="E18" s="41" t="inlineStr">
+        <is>
+          <t>posts every 150, painted green</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="40" t="inlineStr">
+        <is>
+          <t>Skybridge, enclosed tier</t>
+        </is>
+      </c>
+      <c r="B19" s="40" t="inlineStr">
+        <is>
+          <t>500 span</t>
+        </is>
+      </c>
+      <c r="C19" s="40" t="n">
+        <v>300</v>
+      </c>
+      <c r="D19" s="40" t="n">
+        <v>250</v>
+      </c>
+      <c r="E19" s="40" t="inlineStr">
+        <is>
+          <t>underside at about 600 above ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="41" t="inlineStr">
+        <is>
+          <t>Skybridge, girder deck</t>
+        </is>
+      </c>
+      <c r="B20" s="41" t="inlineStr">
+        <is>
+          <t>500 span</t>
+        </is>
+      </c>
+      <c r="C20" s="41" t="n">
+        <v>40</v>
+      </c>
+      <c r="D20" s="41" t="n">
+        <v>250</v>
+      </c>
+      <c r="E20" s="41" t="inlineStr">
+        <is>
+          <t>steel I-beams about 30 deep, sits under the enclosed tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="40" t="inlineStr">
+        <is>
+          <t>Chimney stack</t>
+        </is>
+      </c>
+      <c r="B21" s="40" t="n">
+        <v>180</v>
+      </c>
+      <c r="C21" s="40" t="inlineStr">
+        <is>
+          <t>2800 to top</t>
+        </is>
+      </c>
+      <c r="D21" s="40" t="n">
+        <v>180</v>
+      </c>
+      <c r="E21" s="40" t="inlineStr">
+        <is>
+          <t>top at about 28 m, corbelled cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>Cast-iron drainpipe</t>
+        </is>
+      </c>
+      <c r="B22" s="41" t="inlineStr">
+        <is>
+          <t>10 diameter</t>
+        </is>
+      </c>
+      <c r="C22" s="41" t="inlineStr">
+        <is>
+          <t>full height</t>
+        </is>
+      </c>
+      <c r="D22" s="41" t="n"/>
+      <c r="E22" s="41" t="inlineStr">
+        <is>
+          <t>hopper head 30 x 30, brackets every 180</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="40" t="inlineStr">
+        <is>
+          <t>Plywood sheet</t>
+        </is>
+      </c>
+      <c r="B23" s="40" t="n">
+        <v>122</v>
+      </c>
+      <c r="C23" s="40" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D23" s="40" t="n">
+        <v>244</v>
+      </c>
+      <c r="E23" s="40" t="inlineStr">
+        <is>
+          <t>prop</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="41" t="inlineStr">
+        <is>
+          <t>Timber plank</t>
+        </is>
+      </c>
+      <c r="B24" s="41" t="n">
+        <v>15</v>
+      </c>
+      <c r="C24" s="41" t="n">
+        <v>5</v>
+      </c>
+      <c r="D24" s="41" t="n">
+        <v>240</v>
+      </c>
+      <c r="E24" s="41" t="inlineStr">
+        <is>
+          <t>prop</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="40" t="inlineStr">
+        <is>
+          <t>Ground setts (cobbles)</t>
+        </is>
+      </c>
+      <c r="B25" s="40" t="n">
+        <v>10</v>
+      </c>
+      <c r="C25" s="40" t="n"/>
+      <c r="D25" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="E25" s="40" t="inlineStr">
+        <is>
+          <t>mostly buried under mud and debris</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="42" t="inlineStr">
+        <is>
+          <t>Metrics to hold</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="30" t="inlineStr">
+        <is>
+          <t>Grid snap 25 cm; modules on 100, 200 and 400 cm widths.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="30" t="inlineStr">
+        <is>
+          <t>Floor to floor 400 (left) and 380 (right); pivots at bottom-left-back of each module.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="30" t="inlineStr">
+        <is>
+          <t>Texel density 10.24 px/cm (1024 px/m) for surfaces within 5 m of camera; 5.12 px/cm for upper floors and background.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="30" t="inlineStr">
+        <is>
+          <t>Brick tiling texture covers 200 x 200 cm with 24 courses (8.33 cm each, a small cheat on the real 8.6) so coursing lines up at every 100 cm module edge.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>